<commit_message>
Update TEC22 forecasting checkpoints and direct-model code
</commit_message>
<xml_diff>
--- a/final_predictions_comparison.xlsx
+++ b/final_predictions_comparison.xlsx
@@ -473,7 +473,7 @@
         <v>323.3716667</v>
       </c>
       <c r="B2" t="n">
-        <v>369.0709533691406</v>
+        <v>369.3807983398438</v>
       </c>
       <c r="C2" t="n">
         <v>381.5371861815196</v>
@@ -485,10 +485,10 @@
         <v>374.6404212300389</v>
       </c>
       <c r="F2" t="n">
-        <v>377.3201599121094</v>
+        <v>377.3694152832031</v>
       </c>
       <c r="G2" t="n">
-        <v>375.1932678222656</v>
+        <v>372.3125915527344</v>
       </c>
       <c r="H2" t="n">
         <v>375.2466905028572</v>
@@ -497,7 +497,7 @@
         <v>340.8008810028648</v>
       </c>
       <c r="J2" t="n">
-        <v>329.5840759277344</v>
+        <v>330.4474182128906</v>
       </c>
     </row>
     <row r="3">
@@ -505,7 +505,7 @@
         <v>369.1995833</v>
       </c>
       <c r="B3" t="n">
-        <v>375.1783752441406</v>
+        <v>375.5245666503906</v>
       </c>
       <c r="C3" t="n">
         <v>389.1866013978765</v>
@@ -517,10 +517,10 @@
         <v>383.146895867543</v>
       </c>
       <c r="F3" t="n">
-        <v>380.8391723632812</v>
+        <v>380.9455261230469</v>
       </c>
       <c r="G3" t="n">
-        <v>374.5652465820312</v>
+        <v>372.0897521972656</v>
       </c>
       <c r="H3" t="n">
         <v>381.5918095314288</v>
@@ -529,7 +529,7 @@
         <v>354.8972483054076</v>
       </c>
       <c r="J3" t="n">
-        <v>343.7004699707031</v>
+        <v>344.5498962402344</v>
       </c>
     </row>
     <row r="4">
@@ -537,7 +537,7 @@
         <v>380.0566667</v>
       </c>
       <c r="B4" t="n">
-        <v>376.2181091308594</v>
+        <v>376.570556640625</v>
       </c>
       <c r="C4" t="n">
         <v>390.4865020228783</v>
@@ -549,10 +549,10 @@
         <v>380.8758740108922</v>
       </c>
       <c r="F4" t="n">
-        <v>381.4371643066406</v>
+        <v>381.55322265625</v>
       </c>
       <c r="G4" t="n">
-        <v>374.4585571289062</v>
+        <v>372.039794921875</v>
       </c>
       <c r="H4" t="n">
         <v>380.3260476257144</v>
@@ -561,7 +561,7 @@
         <v>368.0292999233615</v>
       </c>
       <c r="J4" t="n">
-        <v>372.0010986328125</v>
+        <v>372.6620178222656</v>
       </c>
     </row>
     <row r="5">
@@ -569,7 +569,7 @@
         <v>386.9304167</v>
       </c>
       <c r="B5" t="n">
-        <v>377.0182189941406</v>
+        <v>377.37548828125</v>
       </c>
       <c r="C5" t="n">
         <v>391.486425580572</v>
@@ -581,10 +581,10 @@
         <v>382.3213465047481</v>
       </c>
       <c r="F5" t="n">
-        <v>381.8971557617188</v>
+        <v>382.0206909179688</v>
       </c>
       <c r="G5" t="n">
-        <v>374.3764953613281</v>
+        <v>371.9183349609375</v>
       </c>
       <c r="H5" t="n">
         <v>379.7820833400001</v>
@@ -593,7 +593,7 @@
         <v>376.0754858321135</v>
       </c>
       <c r="J5" t="n">
-        <v>379.1035461425781</v>
+        <v>379.7334289550781</v>
       </c>
     </row>
     <row r="6">
@@ -601,7 +601,7 @@
         <v>337.5866667</v>
       </c>
       <c r="B6" t="n">
-        <v>363.657958984375</v>
+        <v>363.9362182617188</v>
       </c>
       <c r="C6" t="n">
         <v>374.7377059892023</v>
@@ -613,10 +613,10 @@
         <v>371.1723033336378</v>
       </c>
       <c r="F6" t="n">
-        <v>374.3056945800781</v>
+        <v>374.4679870605469</v>
       </c>
       <c r="G6" t="n">
-        <v>375.7513427734375</v>
+        <v>372.5107421875</v>
       </c>
       <c r="H6" t="n">
         <v>374.0755595314288</v>
@@ -625,7 +625,7 @@
         <v>373.603354799261</v>
       </c>
       <c r="J6" t="n">
-        <v>382.2680969238281</v>
+        <v>382.7177734375</v>
       </c>
     </row>
     <row r="7">
@@ -633,7 +633,7 @@
         <v>362.9895833</v>
       </c>
       <c r="B7" t="n">
-        <v>365.9247741699219</v>
+        <v>366.2162780761719</v>
       </c>
       <c r="C7" t="n">
         <v>377.5874881286294</v>
@@ -645,10 +645,10 @@
         <v>372.398505118576</v>
       </c>
       <c r="F7" t="n">
-        <v>375.5031433105469</v>
+        <v>375.6156005859375</v>
       </c>
       <c r="G7" t="n">
-        <v>375.5174865722656</v>
+        <v>372.4277038574219</v>
       </c>
       <c r="H7" t="n">
         <v>375.6749404857145</v>
@@ -657,7 +657,7 @@
         <v>349.0725304548834</v>
       </c>
       <c r="J7" t="n">
-        <v>349.7716979980469</v>
+        <v>350.6924743652344</v>
       </c>
     </row>
     <row r="8">
@@ -665,7 +665,7 @@
         <v>370.53375</v>
       </c>
       <c r="B8" t="n">
-        <v>385.96044921875</v>
+        <v>386.3729553222656</v>
       </c>
       <c r="C8" t="n">
         <v>402.635573248857</v>
@@ -677,10 +677,10 @@
         <v>396.3001076489074</v>
       </c>
       <c r="F8" t="n">
-        <v>387.0261840820312</v>
+        <v>387.23291015625</v>
       </c>
       <c r="G8" t="n">
-        <v>372.4668884277344</v>
+        <v>370.5647277832031</v>
       </c>
       <c r="H8" t="n">
         <v>374.7579881028573</v>
@@ -689,7 +689,7 @@
         <v>369.945677231769</v>
       </c>
       <c r="J8" t="n">
-        <v>366.44775390625</v>
+        <v>367.5209045410156</v>
       </c>
     </row>
     <row r="9">
@@ -697,7 +697,7 @@
         <v>376.7820833</v>
       </c>
       <c r="B9" t="n">
-        <v>393.4878234863281</v>
+        <v>393.9482116699219</v>
       </c>
       <c r="C9" t="n">
         <v>411.9848585132932</v>
@@ -709,10 +709,10 @@
         <v>391.3304711172202</v>
       </c>
       <c r="F9" t="n">
-        <v>392.3662719726562</v>
+        <v>392.2640686035156</v>
       </c>
       <c r="G9" t="n">
-        <v>375.9695434570312</v>
+        <v>369.4295349121094</v>
       </c>
       <c r="H9" t="n">
         <v>403.6618333200001</v>
@@ -721,7 +721,7 @@
         <v>386.020769852026</v>
       </c>
       <c r="J9" t="n">
-        <v>378.1078186035156</v>
+        <v>378.587646484375</v>
       </c>
     </row>
     <row r="10">
@@ -729,7 +729,7 @@
         <v>382.8745833</v>
       </c>
       <c r="B10" t="n">
-        <v>390.3046875</v>
+        <v>390.7446899414062</v>
       </c>
       <c r="C10" t="n">
         <v>408.0351604604031</v>
@@ -741,10 +741,10 @@
         <v>391.6519152413453</v>
       </c>
       <c r="F10" t="n">
-        <v>389.5102233886719</v>
+        <v>389.7572021484375</v>
       </c>
       <c r="G10" t="n">
-        <v>373.4657287597656</v>
+        <v>369.9091796875</v>
       </c>
       <c r="H10" t="n">
         <v>391.9562381028571</v>
@@ -753,7 +753,7 @@
         <v>393.0510387758571</v>
       </c>
       <c r="J10" t="n">
-        <v>383.6741638183594</v>
+        <v>383.8713989257812</v>
       </c>
     </row>
     <row r="11">
@@ -761,7 +761,7 @@
         <v>393.5295833</v>
       </c>
       <c r="B11" t="n">
-        <v>385.9202270507812</v>
+        <v>386.3325500488281</v>
       </c>
       <c r="C11" t="n">
         <v>402.5855770709723</v>
@@ -773,10 +773,10 @@
         <v>396.3001076489074</v>
       </c>
       <c r="F11" t="n">
-        <v>387.0032043457031</v>
+        <v>387.2095336914062</v>
       </c>
       <c r="G11" t="n">
-        <v>372.4758605957031</v>
+        <v>370.57080078125</v>
       </c>
       <c r="H11" t="n">
         <v>374.7579881028573</v>
@@ -785,7 +785,7 @@
         <v>387.9849440673034</v>
       </c>
       <c r="J11" t="n">
-        <v>386.4527893066406</v>
+        <v>386.6976928710938</v>
       </c>
     </row>
     <row r="12">
@@ -793,7 +793,7 @@
         <v>390.5954167</v>
       </c>
       <c r="B12" t="n">
-        <v>382.7882690429688</v>
+        <v>383.1809387207031</v>
       </c>
       <c r="C12" t="n">
         <v>398.6858751959668</v>
@@ -805,10 +805,10 @@
         <v>392.7924276345948</v>
       </c>
       <c r="F12" t="n">
-        <v>385.2091979980469</v>
+        <v>385.386474609375</v>
       </c>
       <c r="G12" t="n">
-        <v>373.1757507324219</v>
+        <v>371.0442199707031</v>
       </c>
       <c r="H12" t="n">
         <v>378.1456666857143</v>
@@ -817,7 +817,7 @@
         <v>395.626750904516</v>
       </c>
       <c r="J12" t="n">
-        <v>392.1897888183594</v>
+        <v>392.5216674804688</v>
       </c>
     </row>
     <row r="13">
@@ -825,7 +825,7 @@
         <v>374.0554167</v>
       </c>
       <c r="B13" t="n">
-        <v>386.0408325195312</v>
+        <v>386.4538879394531</v>
       </c>
       <c r="C13" t="n">
         <v>402.7355656046263</v>
@@ -837,10 +837,10 @@
         <v>396.3001076489074</v>
       </c>
       <c r="F13" t="n">
-        <v>387.0722045898438</v>
+        <v>387.2796630859375</v>
       </c>
       <c r="G13" t="n">
-        <v>372.448974609375</v>
+        <v>370.5526123046875</v>
       </c>
       <c r="H13" t="n">
         <v>373.2133928657145</v>
@@ -849,7 +849,7 @@
         <v>386.9897397232332</v>
       </c>
       <c r="J13" t="n">
-        <v>389.3795776367188</v>
+        <v>389.8617248535156</v>
       </c>
     </row>
     <row r="14">
@@ -857,7 +857,7 @@
         <v>449.2825</v>
       </c>
       <c r="B14" t="n">
-        <v>397.4831848144531</v>
+        <v>397.969482421875</v>
       </c>
       <c r="C14" t="n">
         <v>416.9344801238771</v>
@@ -869,10 +869,10 @@
         <v>400.9310117707151</v>
       </c>
       <c r="F14" t="n">
-        <v>396.88525390625</v>
+        <v>396.8113098144531</v>
       </c>
       <c r="G14" t="n">
-        <v>379.1072387695312</v>
+        <v>371.9835510253906</v>
       </c>
       <c r="H14" t="n">
         <v>407.4900357028571</v>
@@ -881,7 +881,7 @@
         <v>395.0830736943475</v>
       </c>
       <c r="J14" t="n">
-        <v>382.3817749023438</v>
+        <v>382.8622741699219</v>
       </c>
     </row>
     <row r="15">
@@ -889,7 +889,7 @@
         <v>541.3645833</v>
       </c>
       <c r="B15" t="n">
-        <v>579.7559814453125</v>
+        <v>581.76513671875</v>
       </c>
       <c r="C15" t="n">
         <v>583.0041939139886</v>
@@ -901,10 +901,10 @@
         <v>570.8680601501321</v>
       </c>
       <c r="F15" t="n">
-        <v>541.720947265625</v>
+        <v>541.9876098632812</v>
       </c>
       <c r="G15" t="n">
-        <v>551.5946044921875</v>
+        <v>548.2138061523438</v>
       </c>
       <c r="H15" t="n">
         <v>583.0497262114286</v>
@@ -913,7 +913,7 @@
         <v>524.0808988300499</v>
       </c>
       <c r="J15" t="n">
-        <v>570.5867309570312</v>
+        <v>569.3720092773438</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         <v>547.5287499999999</v>
       </c>
       <c r="B16" t="n">
-        <v>596.464599609375</v>
+        <v>598.1138305664062</v>
       </c>
       <c r="C16" t="n">
         <v>599.109888126748</v>
@@ -933,10 +933,10 @@
         <v>602.2796592339972</v>
       </c>
       <c r="F16" t="n">
-        <v>574.2916259765625</v>
+        <v>573.9199829101562</v>
       </c>
       <c r="G16" t="n">
-        <v>572.17919921875</v>
+        <v>568.57373046875</v>
       </c>
       <c r="H16" t="n">
         <v>605.5421309571429</v>
@@ -945,7 +945,7 @@
         <v>584.803554058569</v>
       </c>
       <c r="J16" t="n">
-        <v>578.0181274414062</v>
+        <v>577.9220581054688</v>
       </c>
     </row>
     <row r="17">
@@ -953,7 +953,7 @@
         <v>555.3358333</v>
       </c>
       <c r="B17" t="n">
-        <v>594.7621459960938</v>
+        <v>596.3936767578125</v>
       </c>
       <c r="C17" t="n">
         <v>597.1100410113606</v>
@@ -965,10 +965,10 @@
         <v>601.333591182662</v>
       </c>
       <c r="F17" t="n">
-        <v>572.6000366210938</v>
+        <v>572.2341918945312</v>
       </c>
       <c r="G17" t="n">
-        <v>570.4339599609375</v>
+        <v>566.560302734375</v>
       </c>
       <c r="H17" t="n">
         <v>607.2823928514288</v>
@@ -977,7 +977,7 @@
         <v>584.6358870507053</v>
       </c>
       <c r="J17" t="n">
-        <v>578.562744140625</v>
+        <v>578.3850708007812</v>
       </c>
     </row>
     <row r="18">
@@ -985,7 +985,7 @@
         <v>596.44375</v>
       </c>
       <c r="B18" t="n">
-        <v>596.5497436523438</v>
+        <v>598.1997680664062</v>
       </c>
       <c r="C18" t="n">
         <v>599.2098804825174</v>
@@ -997,10 +997,10 @@
         <v>603.7552510285209</v>
       </c>
       <c r="F18" t="n">
-        <v>574.376220703125</v>
+        <v>574.0043334960938</v>
       </c>
       <c r="G18" t="n">
-        <v>572.26025390625</v>
+        <v>568.674560546875</v>
       </c>
       <c r="H18" t="n">
         <v>605.5421309571429</v>
@@ -1009,7 +1009,7 @@
         <v>579.7704417964934</v>
       </c>
       <c r="J18" t="n">
-        <v>580.5171508789062</v>
+        <v>580.4696655273438</v>
       </c>
     </row>
     <row r="19">
@@ -1017,7 +1017,7 @@
         <v>568.0754167</v>
       </c>
       <c r="B19" t="n">
-        <v>598.3803100585938</v>
+        <v>600.0493774414062</v>
       </c>
       <c r="C19" t="n">
         <v>601.3597161315589</v>
@@ -1029,10 +1029,10 @@
         <v>603.3334172139281</v>
       </c>
       <c r="F19" t="n">
-        <v>576.3271484375</v>
+        <v>575.8165893554688</v>
       </c>
       <c r="G19" t="n">
-        <v>574.0031127929688</v>
+        <v>570.8386840820312</v>
       </c>
       <c r="H19" t="n">
         <v>609.9228690514286</v>
@@ -1041,7 +1041,7 @@
         <v>604.083096743692</v>
       </c>
       <c r="J19" t="n">
-        <v>600.6173095703125</v>
+        <v>600.8052978515625</v>
       </c>
     </row>
     <row r="20">
@@ -1049,7 +1049,7 @@
         <v>588.1533333</v>
       </c>
       <c r="B20" t="n">
-        <v>585.7867431640625</v>
+        <v>587.3267211914062</v>
       </c>
       <c r="C20" t="n">
         <v>586.5608474776919</v>
@@ -1061,10 +1061,10 @@
         <v>590.6550575435035</v>
       </c>
       <c r="F20" t="n">
-        <v>563.6767578125</v>
+        <v>563.3413696289062</v>
       </c>
       <c r="G20" t="n">
-        <v>561.0994262695312</v>
+        <v>555.939453125</v>
       </c>
       <c r="H20" t="n">
         <v>609.3331785857143</v>
@@ -1073,7 +1073,7 @@
         <v>583.2262832587509</v>
       </c>
       <c r="J20" t="n">
-        <v>581.3887939453125</v>
+        <v>581.1903076171875</v>
       </c>
     </row>
     <row r="21">
@@ -1081,7 +1081,7 @@
         <v>691.8041667</v>
       </c>
       <c r="B21" t="n">
-        <v>580.7716674804688</v>
+        <v>582.2612915039062</v>
       </c>
       <c r="C21" t="n">
         <v>580.6612984872991</v>
@@ -1093,10 +1093,10 @@
         <v>578.0082019068008</v>
       </c>
       <c r="F21" t="n">
-        <v>558.6864624023438</v>
+        <v>558.3681640625</v>
       </c>
       <c r="G21" t="n">
-        <v>555.8792114257812</v>
+        <v>550</v>
       </c>
       <c r="H21" t="n">
         <v>629.64085714</v>
@@ -1105,7 +1105,7 @@
         <v>589.2443628069228</v>
       </c>
       <c r="J21" t="n">
-        <v>585.450927734375</v>
+        <v>585.4951782226562</v>
       </c>
     </row>
     <row r="22">
@@ -1113,7 +1113,7 @@
         <v>712.31875</v>
       </c>
       <c r="B22" t="n">
-        <v>759.7312622070312</v>
+        <v>761.02880859375</v>
       </c>
       <c r="C22" t="n">
         <v>748.1066824464144</v>
@@ -1125,10 +1125,10 @@
         <v>740.1623689942055</v>
       </c>
       <c r="F22" t="n">
-        <v>738.1602783203125</v>
+        <v>740.2860717773438</v>
       </c>
       <c r="G22" t="n">
-        <v>778.3395385742188</v>
+        <v>780.3607788085938</v>
       </c>
       <c r="H22" t="n">
         <v>733.3346785685717</v>
@@ -1137,7 +1137,7 @@
         <v>729.0358277655029</v>
       </c>
       <c r="J22" t="n">
-        <v>776.9022216796875</v>
+        <v>774.3435668945312</v>
       </c>
     </row>
     <row r="23">
@@ -1145,7 +1145,7 @@
         <v>584.9425</v>
       </c>
       <c r="B23" t="n">
-        <v>584.1332397460938</v>
+        <v>584.361328125</v>
       </c>
       <c r="C23" t="n">
         <v>581.5370068774561</v>
@@ -1157,10 +1157,10 @@
         <v>565.5138111390341</v>
       </c>
       <c r="F23" t="n">
-        <v>542.2236938476562</v>
+        <v>542.458251953125</v>
       </c>
       <c r="G23" t="n">
-        <v>571.412841796875</v>
+        <v>569.6159057617188</v>
       </c>
       <c r="H23" t="n">
         <v>613.5544166571427</v>
@@ -1169,7 +1169,7 @@
         <v>615.2486594622574</v>
       </c>
       <c r="J23" t="n">
-        <v>570.8951416015625</v>
+        <v>571.26025390625</v>
       </c>
     </row>
     <row r="24">
@@ -1177,7 +1177,7 @@
         <v>571.2483333</v>
       </c>
       <c r="B24" t="n">
-        <v>583</v>
+        <v>583.2193603515625</v>
       </c>
       <c r="C24" t="n">
         <v>580.2371062524542</v>
@@ -1189,10 +1189,10 @@
         <v>561.6296005296341</v>
       </c>
       <c r="F24" t="n">
-        <v>541.4263305664062</v>
+        <v>541.6640625</v>
       </c>
       <c r="G24" t="n">
-        <v>570.493408203125</v>
+        <v>568.6453857421875</v>
       </c>
       <c r="H24" t="n">
         <v>613.2011666685714</v>
@@ -1201,7 +1201,7 @@
         <v>584.8067851978001</v>
       </c>
       <c r="J24" t="n">
-        <v>574.6317138671875</v>
+        <v>575.7731323242188</v>
       </c>
     </row>
     <row r="25">
@@ -1209,7 +1209,7 @@
         <v>536.4108333</v>
       </c>
       <c r="B25" t="n">
-        <v>586.35693359375</v>
+        <v>586.6024169921875</v>
       </c>
       <c r="C25" t="n">
         <v>584.086811949575</v>
@@ -1221,10 +1221,10 @@
         <v>576.7338890356272</v>
       </c>
       <c r="F25" t="n">
-        <v>543.7877197265625</v>
+        <v>544.0162353515625</v>
       </c>
       <c r="G25" t="n">
-        <v>573.0718994140625</v>
+        <v>571.6322021484375</v>
       </c>
       <c r="H25" t="n">
         <v>573.8100416671429</v>
@@ -1233,7 +1233,7 @@
         <v>575.7952427830083</v>
       </c>
       <c r="J25" t="n">
-        <v>566.7742309570312</v>
+        <v>568.00390625</v>
       </c>
     </row>
     <row r="26">
@@ -1241,7 +1241,7 @@
         <v>584.05375</v>
       </c>
       <c r="B26" t="n">
-        <v>591.1567993164062</v>
+        <v>591.440185546875</v>
       </c>
       <c r="C26" t="n">
         <v>589.5863915168904</v>
@@ -1253,10 +1253,10 @@
         <v>594.3594359837433</v>
       </c>
       <c r="F26" t="n">
-        <v>547.1611328125</v>
+        <v>547.37646484375</v>
       </c>
       <c r="G26" t="n">
-        <v>576.6503295898438</v>
+        <v>576.0721435546875</v>
       </c>
       <c r="H26" t="n">
         <v>651.1492142942857</v>
@@ -1265,7 +1265,7 @@
         <v>559.8758059861985</v>
       </c>
       <c r="J26" t="n">
-        <v>547.8148193359375</v>
+        <v>548.9656372070312</v>
       </c>
     </row>
     <row r="27">
@@ -1273,7 +1273,7 @@
         <v>566.3595833000001</v>
       </c>
       <c r="B27" t="n">
-        <v>598.1474609375</v>
+        <v>598.487060546875</v>
       </c>
       <c r="C27" t="n">
         <v>597.5857799784402</v>
@@ -1285,10 +1285,10 @@
         <v>601.5459842576206</v>
       </c>
       <c r="F27" t="n">
-        <v>552.0679321289062</v>
+        <v>552.26416015625</v>
       </c>
       <c r="G27" t="n">
-        <v>581.8551635742188</v>
+        <v>582.5227661132812</v>
       </c>
       <c r="H27" t="n">
         <v>606.3200119114285</v>
@@ -1297,7 +1297,7 @@
         <v>592.7147942524921</v>
       </c>
       <c r="J27" t="n">
-        <v>579.2664184570312</v>
+        <v>580.3298950195312</v>
       </c>
     </row>
     <row r="28">
@@ -1305,7 +1305,7 @@
         <v>591.7333333</v>
       </c>
       <c r="B28" t="n">
-        <v>603.397216796875</v>
+        <v>603.7794799804688</v>
       </c>
       <c r="C28" t="n">
         <v>603.5853213246025</v>
@@ -1317,10 +1317,10 @@
         <v>614.0647744818754</v>
       </c>
       <c r="F28" t="n">
-        <v>555.858154296875</v>
+        <v>555.9751586914062</v>
       </c>
       <c r="G28" t="n">
-        <v>585.8838500976562</v>
+        <v>587.2156982421875</v>
       </c>
       <c r="H28" t="n">
         <v>614.9166785885715</v>
@@ -1329,7 +1329,7 @@
         <v>587.2637812215072</v>
       </c>
       <c r="J28" t="n">
-        <v>572.0264892578125</v>
+        <v>572.9999389648438</v>
       </c>
     </row>
     <row r="29">
@@ -1337,7 +1337,7 @@
         <v>587.0004167</v>
       </c>
       <c r="B29" t="n">
-        <v>603.572265625</v>
+        <v>603.9559936523438</v>
       </c>
       <c r="C29" t="n">
         <v>603.7853060361413</v>
@@ -1349,10 +1349,10 @@
         <v>612.9264861842025</v>
       </c>
       <c r="F29" t="n">
-        <v>555.9864501953125</v>
+        <v>556.1045532226562</v>
       </c>
       <c r="G29" t="n">
-        <v>586.0205078125</v>
+        <v>587.3721313476562</v>
       </c>
       <c r="H29" t="n">
         <v>615.1450952542858</v>
@@ -1361,7 +1361,7 @@
         <v>602.6164927079751</v>
       </c>
       <c r="J29" t="n">
-        <v>591.6967163085938</v>
+        <v>592.4320678710938</v>
       </c>
     </row>
     <row r="30">
@@ -1369,7 +1369,7 @@
         <v>605.9974999999999</v>
       </c>
       <c r="B30" t="n">
-        <v>602.1716918945312</v>
+        <v>602.5440673828125</v>
       </c>
       <c r="C30" t="n">
         <v>602.1854283438313</v>
@@ -1381,10 +1381,10 @@
         <v>614.8745968618671</v>
       </c>
       <c r="F30" t="n">
-        <v>554.9597778320312</v>
+        <v>555.0745239257812</v>
       </c>
       <c r="G30" t="n">
-        <v>584.9269409179688</v>
+        <v>586.1207275390625</v>
       </c>
       <c r="H30" t="n">
         <v>636.5122381114286</v>
@@ -1393,7 +1393,7 @@
         <v>597.9847871633623</v>
       </c>
       <c r="J30" t="n">
-        <v>587.2252807617188</v>
+        <v>588.009765625</v>
       </c>
     </row>
     <row r="31">
@@ -1401,7 +1401,7 @@
         <v>630.1970833</v>
       </c>
       <c r="B31" t="n">
-        <v>594.7819213867188</v>
+        <v>595.0942993164062</v>
       </c>
       <c r="C31" t="n">
         <v>593.7360742813194</v>
@@ -1413,10 +1413,10 @@
         <v>590.1710044964142</v>
       </c>
       <c r="F31" t="n">
-        <v>549.70654296875</v>
+        <v>549.9119873046875</v>
       </c>
       <c r="G31" t="n">
-        <v>579.3504028320312</v>
+        <v>579.4222412109375</v>
       </c>
       <c r="H31" t="n">
         <v>619.2266428514286</v>
@@ -1425,7 +1425,7 @@
         <v>612.2326127791282</v>
       </c>
       <c r="J31" t="n">
-        <v>597.728271484375</v>
+        <v>598.4472045898438</v>
       </c>
     </row>
     <row r="32">
@@ -1433,7 +1433,7 @@
         <v>597.6070833</v>
       </c>
       <c r="B32" t="n">
-        <v>603.4055786132812</v>
+        <v>605.126953125</v>
       </c>
       <c r="C32" t="n">
         <v>607.2592651219518</v>
@@ -1445,10 +1445,10 @@
         <v>607.9623022595102</v>
       </c>
       <c r="F32" t="n">
-        <v>581.6980590820312</v>
+        <v>580.7898559570312</v>
       </c>
       <c r="G32" t="n">
-        <v>578.7859497070312</v>
+        <v>576.449462890625</v>
       </c>
       <c r="H32" t="n">
         <v>591.9098095257143</v>
@@ -1457,7 +1457,7 @@
         <v>604.0720593726995</v>
       </c>
       <c r="J32" t="n">
-        <v>609.0259399414062</v>
+        <v>608.7622680664062</v>
       </c>
     </row>
     <row r="33">
@@ -1465,7 +1465,7 @@
         <v>589.4229167</v>
       </c>
       <c r="B33" t="n">
-        <v>607.96435546875</v>
+        <v>609.7338256835938</v>
       </c>
       <c r="C33" t="n">
         <v>612.6088561556132</v>
@@ -1477,10 +1477,10 @@
         <v>619.5842084890899</v>
       </c>
       <c r="F33" t="n">
-        <v>586.5682983398438</v>
+        <v>585.82373046875</v>
       </c>
       <c r="G33" t="n">
-        <v>583.1229858398438</v>
+        <v>581.40380859375</v>
       </c>
       <c r="H33" t="n">
         <v>623.1732619200001</v>
@@ -1489,7 +1489,7 @@
         <v>607.0914657306907</v>
       </c>
       <c r="J33" t="n">
-        <v>605.9783935546875</v>
+        <v>606.0927734375</v>
       </c>
     </row>
     <row r="34">
@@ -1497,7 +1497,7 @@
         <v>587.1458333</v>
       </c>
       <c r="B34" t="n">
-        <v>607.4956665039062</v>
+        <v>609.2601318359375</v>
       </c>
       <c r="C34" t="n">
         <v>612.0588981988817</v>
@@ -1509,10 +1509,10 @@
         <v>617.5379048797248</v>
       </c>
       <c r="F34" t="n">
-        <v>586.0675659179688</v>
+        <v>585.2278442382812</v>
       </c>
       <c r="G34" t="n">
-        <v>582.6770629882812</v>
+        <v>580.8944702148438</v>
       </c>
       <c r="H34" t="n">
         <v>617.9314404828572</v>
@@ -1521,7 +1521,7 @@
         <v>605.4998998162359</v>
       </c>
       <c r="J34" t="n">
-        <v>602.5159301757812</v>
+        <v>602.5574340820312</v>
       </c>
     </row>
     <row r="35">
@@ -1529,7 +1529,7 @@
         <v>598.4866667</v>
       </c>
       <c r="B35" t="n">
-        <v>597.0606079101562</v>
+        <v>598.7158813476562</v>
       </c>
       <c r="C35" t="n">
         <v>599.8098346171337</v>
@@ -1541,10 +1541,10 @@
         <v>604.0622427263718</v>
       </c>
       <c r="F35" t="n">
-        <v>574.9161376953125</v>
+        <v>574.5101318359375</v>
       </c>
       <c r="G35" t="n">
-        <v>572.74658203125</v>
+        <v>569.2784423828125</v>
       </c>
       <c r="H35" t="n">
         <v>606.9742023857143</v>
@@ -1553,7 +1553,7 @@
         <v>601.967483664726</v>
       </c>
       <c r="J35" t="n">
-        <v>598.1239624023438</v>
+        <v>598.0015258789062</v>
       </c>
     </row>
     <row r="36">
@@ -1561,7 +1561,7 @@
         <v>522.7141667</v>
       </c>
       <c r="B36" t="n">
-        <v>595.0173950195312</v>
+        <v>596.6516723632812</v>
       </c>
       <c r="C36" t="n">
         <v>597.4100180786688</v>
@@ -1573,10 +1573,10 @@
         <v>601.333591182662</v>
       </c>
       <c r="F36" t="n">
-        <v>572.853759765625</v>
+        <v>572.4871215820312</v>
       </c>
       <c r="G36" t="n">
-        <v>570.6993408203125</v>
+        <v>566.8622436523438</v>
       </c>
       <c r="H36" t="n">
         <v>606.4027857142859</v>
@@ -1585,7 +1585,7 @@
         <v>604.5021685484652</v>
       </c>
       <c r="J36" t="n">
-        <v>600.4688720703125</v>
+        <v>600.55029296875</v>
       </c>
     </row>
     <row r="37">
@@ -1593,7 +1593,7 @@
         <v>606.4766667</v>
       </c>
       <c r="B37" t="n">
-        <v>604.8113403320312</v>
+        <v>606.5474853515625</v>
       </c>
       <c r="C37" t="n">
         <v>608.9091389921465</v>
@@ -1605,10 +1605,10 @@
         <v>616.0138573570542</v>
       </c>
       <c r="F37" t="n">
-        <v>583.2000122070312</v>
+        <v>582.2913208007812</v>
       </c>
       <c r="G37" t="n">
-        <v>580.1236572265625</v>
+        <v>577.9774169921875</v>
       </c>
       <c r="H37" t="n">
         <v>596.3613333485714</v>
@@ -1617,7 +1617,7 @@
         <v>553.9440609470146</v>
       </c>
       <c r="J37" t="n">
-        <v>558.3843994140625</v>
+        <v>558.6663818359375</v>
       </c>
     </row>
     <row r="38">
@@ -1625,7 +1625,7 @@
         <v>605.8154167</v>
       </c>
       <c r="B38" t="n">
-        <v>595.3153686523438</v>
+        <v>596.9526977539062</v>
       </c>
       <c r="C38" t="n">
         <v>597.7599913238615</v>
@@ -1637,10 +1637,10 @@
         <v>601.2811559424679</v>
       </c>
       <c r="F38" t="n">
-        <v>573.1497802734375</v>
+        <v>572.7821655273438</v>
       </c>
       <c r="G38" t="n">
-        <v>571.009033203125</v>
+        <v>567.2147216796875</v>
       </c>
       <c r="H38" t="n">
         <v>608.8655119028573</v>
@@ -1649,7 +1649,7 @@
         <v>613.6610052236857</v>
       </c>
       <c r="J38" t="n">
-        <v>608.1448364257812</v>
+        <v>608.05029296875</v>
       </c>
     </row>
     <row r="39">
@@ -1657,7 +1657,7 @@
         <v>602.165</v>
       </c>
       <c r="B39" t="n">
-        <v>595.35791015625</v>
+        <v>596.9956665039062</v>
       </c>
       <c r="C39" t="n">
         <v>597.8099875017463</v>
@@ -1669,10 +1669,10 @@
         <v>601.2811559424679</v>
       </c>
       <c r="F39" t="n">
-        <v>573.192138671875</v>
+        <v>572.82421875</v>
       </c>
       <c r="G39" t="n">
-        <v>571.0531616210938</v>
+        <v>567.264892578125</v>
       </c>
       <c r="H39" t="n">
         <v>608.8655119028573</v>
@@ -1681,7 +1681,7 @@
         <v>610.1414719356129</v>
       </c>
       <c r="J39" t="n">
-        <v>602.9412231445312</v>
+        <v>603.0863647460938</v>
       </c>
     </row>
     <row r="40">
@@ -1689,7 +1689,7 @@
         <v>586.0225</v>
       </c>
       <c r="B40" t="n">
-        <v>581.748779296875</v>
+        <v>583.2482299804688</v>
       </c>
       <c r="C40" t="n">
         <v>581.8112105786468</v>
@@ -1701,10 +1701,10 @@
         <v>582.0007859036124</v>
       </c>
       <c r="F40" t="n">
-        <v>559.6591796875</v>
+        <v>559.3374633789062</v>
       </c>
       <c r="G40" t="n">
-        <v>556.896728515625</v>
+        <v>551.1575927734375</v>
       </c>
       <c r="H40" t="n">
         <v>624.6710357114287</v>
@@ -1713,7 +1713,7 @@
         <v>601.3371758768744</v>
       </c>
       <c r="J40" t="n">
-        <v>597.0468139648438</v>
+        <v>596.9744262695312</v>
       </c>
     </row>
     <row r="41">
@@ -1721,7 +1721,7 @@
         <v>575.59</v>
       </c>
       <c r="B41" t="n">
-        <v>584.2138061523438</v>
+        <v>585.7379150390625</v>
       </c>
       <c r="C41" t="n">
         <v>584.7109888959585</v>
@@ -1733,10 +1733,10 @@
         <v>587.7146398959397</v>
       </c>
       <c r="F41" t="n">
-        <v>562.1119995117188</v>
+        <v>561.7819213867188</v>
       </c>
       <c r="G41" t="n">
-        <v>559.4625244140625</v>
+        <v>554.0771484375</v>
       </c>
       <c r="H41" t="n">
         <v>614.5988809628573</v>
@@ -1745,7 +1745,7 @@
         <v>585.3183810527287</v>
       </c>
       <c r="J41" t="n">
-        <v>583.0711059570312</v>
+        <v>583.3441772460938</v>
       </c>
     </row>
     <row r="42">
@@ -1753,7 +1753,7 @@
         <v>583.4241667</v>
       </c>
       <c r="B42" t="n">
-        <v>590.0392456054688</v>
+        <v>591.6224365234375</v>
       </c>
       <c r="C42" t="n">
         <v>591.5604652661605</v>
@@ -1765,10 +1765,10 @@
         <v>587.4021496346654</v>
       </c>
       <c r="F42" t="n">
-        <v>567.90576171875</v>
+        <v>567.5559692382812</v>
       </c>
       <c r="G42" t="n">
-        <v>565.5233764648438</v>
+        <v>560.9730224609375</v>
       </c>
       <c r="H42" t="n">
         <v>603.8341309628571</v>
@@ -1777,7 +1777,7 @@
         <v>581.1661385649219</v>
       </c>
       <c r="J42" t="n">
-        <v>579.27197265625</v>
+        <v>579.5728759765625</v>
       </c>
     </row>
     <row r="43">
@@ -1785,7 +1785,7 @@
         <v>588.7925</v>
       </c>
       <c r="B43" t="n">
-        <v>594.591796875</v>
+        <v>596.2216796875</v>
       </c>
       <c r="C43" t="n">
         <v>596.9100562998219</v>
@@ -1797,10 +1797,10 @@
         <v>601.3200478628391</v>
       </c>
       <c r="F43" t="n">
-        <v>572.4308471679688</v>
+        <v>572.0655517578125</v>
       </c>
       <c r="G43" t="n">
-        <v>570.2570190429688</v>
+        <v>566.35888671875</v>
       </c>
       <c r="H43" t="n">
         <v>607.2194166571431</v>
@@ -1809,7 +1809,7 @@
         <v>593.0432737197779</v>
       </c>
       <c r="J43" t="n">
-        <v>588.0748901367188</v>
+        <v>588.28662109375</v>
       </c>
     </row>
     <row r="44">
@@ -1817,7 +1817,7 @@
         <v>593.7595833</v>
       </c>
       <c r="B44" t="n">
-        <v>594.5491943359375</v>
+        <v>596.1787719726562</v>
       </c>
       <c r="C44" t="n">
         <v>596.8600601219372</v>
@@ -1829,10 +1829,10 @@
         <v>601.3200478628391</v>
       </c>
       <c r="F44" t="n">
-        <v>572.3886108398438</v>
+        <v>572.0234985351562</v>
       </c>
       <c r="G44" t="n">
-        <v>570.212646484375</v>
+        <v>566.30859375</v>
       </c>
       <c r="H44" t="n">
         <v>607.2194166571431</v>
@@ -1841,7 +1841,7 @@
         <v>598.2730119311137</v>
       </c>
       <c r="J44" t="n">
-        <v>593.764404296875</v>
+        <v>593.8348999023438</v>
       </c>
     </row>
     <row r="45">
@@ -1849,7 +1849,7 @@
         <v>588.9133333</v>
       </c>
       <c r="B45" t="n">
-        <v>593.5278930664062</v>
+        <v>595.1469116210938</v>
       </c>
       <c r="C45" t="n">
         <v>595.6601518527048</v>
@@ -1861,10 +1861,10 @@
         <v>595.825923323762</v>
       </c>
       <c r="F45" t="n">
-        <v>571.3735961914062</v>
+        <v>571.011962890625</v>
       </c>
       <c r="G45" t="n">
-        <v>569.1510009765625</v>
+        <v>565.1005249023438</v>
       </c>
       <c r="H45" t="n">
         <v>606.5617380857145</v>
@@ -1873,7 +1873,7 @@
         <v>598.5096897433673</v>
       </c>
       <c r="J45" t="n">
-        <v>595.99658203125</v>
+        <v>596.0838012695312</v>
       </c>
     </row>
     <row r="46">
@@ -1881,7 +1881,7 @@
         <v>519.9558333</v>
       </c>
       <c r="B46" t="n">
-        <v>594.591796875</v>
+        <v>596.2216796875</v>
       </c>
       <c r="C46" t="n">
         <v>596.9100562998219</v>
@@ -1893,10 +1893,10 @@
         <v>601.3200478628391</v>
       </c>
       <c r="F46" t="n">
-        <v>572.4308471679688</v>
+        <v>572.0655517578125</v>
       </c>
       <c r="G46" t="n">
-        <v>570.2570190429688</v>
+        <v>566.35888671875</v>
       </c>
       <c r="H46" t="n">
         <v>607.2194166571431</v>
@@ -1905,7 +1905,7 @@
         <v>598.4871047690878</v>
       </c>
       <c r="J46" t="n">
-        <v>593.370849609375</v>
+        <v>593.5262451171875</v>
       </c>
     </row>
     <row r="47">
@@ -1913,7 +1913,7 @@
         <v>553.8358333</v>
       </c>
       <c r="B47" t="n">
-        <v>612.2750244140625</v>
+        <v>613.4049682617188</v>
       </c>
       <c r="C47" t="n">
         <v>613.5206160284997</v>
@@ -1925,10 +1925,10 @@
         <v>598.5326557179978</v>
       </c>
       <c r="F47" t="n">
-        <v>602.46044921875</v>
+        <v>601.508544921875</v>
       </c>
       <c r="G47" t="n">
-        <v>590.7554931640625</v>
+        <v>582.5433959960938</v>
       </c>
       <c r="H47" t="n">
         <v>579.1138571457143</v>
@@ -1937,7 +1937,7 @@
         <v>562.5785863731606</v>
       </c>
       <c r="J47" t="n">
-        <v>555.8778076171875</v>
+        <v>555.795654296875</v>
       </c>
     </row>
     <row r="48">
@@ -1945,7 +1945,7 @@
         <v>553.8595833000001</v>
       </c>
       <c r="B48" t="n">
-        <v>611.8034057617188</v>
+        <v>612.9283447265625</v>
       </c>
       <c r="C48" t="n">
         <v>612.9706580717682</v>
@@ -1957,10 +1957,10 @@
         <v>598.2200828558987</v>
       </c>
       <c r="F48" t="n">
-        <v>601.9609375</v>
+        <v>601.0067138671875</v>
       </c>
       <c r="G48" t="n">
-        <v>590.17626953125</v>
+        <v>581.8922729492188</v>
       </c>
       <c r="H48" t="n">
         <v>551.4995714457144</v>
@@ -1969,7 +1969,7 @@
         <v>576.4560480979719</v>
       </c>
       <c r="J48" t="n">
-        <v>574.2946166992188</v>
+        <v>574.1953125</v>
       </c>
     </row>
     <row r="49">
@@ -1977,7 +1977,7 @@
         <v>567.8054167</v>
       </c>
       <c r="B49" t="n">
-        <v>607.344970703125</v>
+        <v>608.42431640625</v>
       </c>
       <c r="C49" t="n">
         <v>607.7710555717608</v>
@@ -1989,10 +1989,10 @@
         <v>588.5832803214521</v>
       </c>
       <c r="F49" t="n">
-        <v>597.2383422851562</v>
+        <v>596.2619018554688</v>
       </c>
       <c r="G49" t="n">
-        <v>584.70068359375</v>
+        <v>575.7379760742188</v>
       </c>
       <c r="H49" t="n">
         <v>570.26657144</v>
@@ -2001,7 +2001,7 @@
         <v>576.4957235219231</v>
       </c>
       <c r="J49" t="n">
-        <v>570.6531982421875</v>
+        <v>570.5993041992188</v>
       </c>
     </row>
     <row r="50">
@@ -2009,7 +2009,7 @@
         <v>590.2958333</v>
       </c>
       <c r="B50" t="n">
-        <v>606.9164428710938</v>
+        <v>607.9913330078125</v>
       </c>
       <c r="C50" t="n">
         <v>607.2710937929139</v>
@@ -2021,10 +2021,10 @@
         <v>586.1662483055563</v>
       </c>
       <c r="F50" t="n">
-        <v>596.7842407226562</v>
+        <v>595.8057250976562</v>
       </c>
       <c r="G50" t="n">
-        <v>584.1741943359375</v>
+        <v>575.1461791992188</v>
       </c>
       <c r="H50" t="n">
         <v>570.2724881057144</v>
@@ -2033,7 +2033,7 @@
         <v>582.8816714889456</v>
       </c>
       <c r="J50" t="n">
-        <v>576.0527954101562</v>
+        <v>576.1232299804688</v>
       </c>
     </row>
     <row r="51">
@@ -2041,7 +2041,7 @@
         <v>579.8716667</v>
       </c>
       <c r="B51" t="n">
-        <v>599.0762329101562</v>
+        <v>600.072021484375</v>
       </c>
       <c r="C51" t="n">
         <v>598.1217932400165</v>
@@ -2053,10 +2053,10 @@
         <v>579.8066034881148</v>
       </c>
       <c r="F51" t="n">
-        <v>588.4743041992188</v>
+        <v>587.4567260742188</v>
       </c>
       <c r="G51" t="n">
-        <v>574.539306640625</v>
+        <v>565.876708984375</v>
       </c>
       <c r="H51" t="n">
         <v>595.7697500028572</v>
@@ -2065,7 +2065,7 @@
         <v>592.3943548382728</v>
       </c>
       <c r="J51" t="n">
-        <v>587.9890747070312</v>
+        <v>587.9051513671875</v>
       </c>
     </row>
     <row r="52">
@@ -2073,7 +2073,7 @@
         <v>682.8316667</v>
       </c>
       <c r="B52" t="n">
-        <v>599.9755859375</v>
+        <v>600.9804077148438</v>
       </c>
       <c r="C52" t="n">
         <v>599.1717129755949</v>
@@ -2085,10 +2085,10 @@
         <v>584.6139265315013</v>
       </c>
       <c r="F52" t="n">
-        <v>589.4278564453125</v>
+        <v>588.4148559570312</v>
       </c>
       <c r="G52" t="n">
-        <v>575.6449584960938</v>
+        <v>566.9204711914062</v>
       </c>
       <c r="H52" t="n">
         <v>579.2713571542857</v>
@@ -2097,7 +2097,7 @@
         <v>579.8730441941003</v>
       </c>
       <c r="J52" t="n">
-        <v>577.5325927734375</v>
+        <v>577.6446533203125</v>
       </c>
     </row>
     <row r="53">
@@ -2105,7 +2105,7 @@
         <v>589.3829167</v>
       </c>
       <c r="B53" t="n">
-        <v>607.8873291015625</v>
+        <v>607.6500854492188</v>
       </c>
       <c r="C53" t="n">
         <v>604.0471155965269</v>
@@ -2117,10 +2117,10 @@
         <v>598.5211081090922</v>
       </c>
       <c r="F53" t="n">
-        <v>596.2076416015625</v>
+        <v>597.0013427734375</v>
       </c>
       <c r="G53" t="n">
-        <v>594.1051025390625</v>
+        <v>591.106689453125</v>
       </c>
       <c r="H53" t="n">
         <v>624.366</v>
@@ -2129,7 +2129,7 @@
         <v>608.361312784753</v>
       </c>
       <c r="J53" t="n">
-        <v>615.1419067382812</v>
+        <v>612.5582275390625</v>
       </c>
     </row>
     <row r="54">
@@ -2137,7 +2137,7 @@
         <v>542.9475</v>
       </c>
       <c r="B54" t="n">
-        <v>616.892578125</v>
+        <v>616.727294921875</v>
       </c>
       <c r="C54" t="n">
         <v>614.2463358850027</v>
@@ -2149,10 +2149,10 @@
         <v>614.2656733231631</v>
       </c>
       <c r="F54" t="n">
-        <v>602.4638061523438</v>
+        <v>603.2330932617188</v>
       </c>
       <c r="G54" t="n">
-        <v>601.4931030273438</v>
+        <v>599.2952880859375</v>
       </c>
       <c r="H54" t="n">
         <v>594.1654166628572</v>
@@ -2161,7 +2161,7 @@
         <v>588.9170138331835</v>
       </c>
       <c r="J54" t="n">
-        <v>583.0801391601562</v>
+        <v>584.1436157226562</v>
       </c>
     </row>
     <row r="55">
@@ -2169,7 +2169,7 @@
         <v>591.8441667</v>
       </c>
       <c r="B55" t="n">
-        <v>615.1256713867188</v>
+        <v>614.9461669921875</v>
       </c>
       <c r="C55" t="n">
         <v>612.2464887696153</v>
@@ -2181,10 +2181,10 @@
         <v>601.4355173115737</v>
       </c>
       <c r="F55" t="n">
-        <v>601.2371215820312</v>
+        <v>602.0111694335938</v>
       </c>
       <c r="G55" t="n">
-        <v>600.0445556640625</v>
+        <v>597.8018798828125</v>
       </c>
       <c r="H55" t="n">
         <v>577.8277142885717</v>
@@ -2193,7 +2193,7 @@
         <v>570.9628530535573</v>
       </c>
       <c r="J55" t="n">
-        <v>558.9456787109375</v>
+        <v>559.8225708007812</v>
       </c>
     </row>
     <row r="56">
@@ -2201,7 +2201,7 @@
         <v>589.6675</v>
       </c>
       <c r="B56" t="n">
-        <v>624.8944702148438</v>
+        <v>624.794677734375</v>
       </c>
       <c r="C56" t="n">
         <v>623.2956440821308</v>
@@ -2213,10 +2213,10 @@
         <v>622.205163493007</v>
       </c>
       <c r="F56" t="n">
-        <v>608.0145874023438</v>
+        <v>608.7622680664062</v>
       </c>
       <c r="G56" t="n">
-        <v>607.697998046875</v>
+        <v>606.0523681640625</v>
       </c>
       <c r="H56" t="n">
         <v>627.7054404771429</v>
@@ -2225,7 +2225,7 @@
         <v>604.0716181190061</v>
       </c>
       <c r="J56" t="n">
-        <v>590.5310668945312</v>
+        <v>591.4541015625</v>
       </c>
     </row>
     <row r="57">
@@ -2233,7 +2233,7 @@
         <v>594.3049999999999</v>
       </c>
       <c r="B57" t="n">
-        <v>624.3193969726562</v>
+        <v>624.2147827148438</v>
       </c>
       <c r="C57" t="n">
         <v>622.6456937696299</v>
@@ -2245,10 +2245,10 @@
         <v>622.2215211151758</v>
       </c>
       <c r="F57" t="n">
-        <v>607.615966796875</v>
+        <v>608.3651123046875</v>
       </c>
       <c r="G57" t="n">
-        <v>607.2695922851562</v>
+        <v>605.5670776367188</v>
       </c>
       <c r="H57" t="n">
         <v>627.7054404771429</v>
@@ -2257,7 +2257,7 @@
         <v>606.3199044944669</v>
       </c>
       <c r="J57" t="n">
-        <v>593.0051879882812</v>
+        <v>593.6860961914062</v>
       </c>
     </row>
     <row r="58">
@@ -2265,7 +2265,7 @@
         <v>590.6120833</v>
       </c>
       <c r="B58" t="n">
-        <v>619.63232421875</v>
+        <v>619.4893188476562</v>
       </c>
       <c r="C58" t="n">
         <v>617.3460989138532</v>
@@ -2277,10 +2277,10 @@
         <v>618.4101129405277</v>
       </c>
       <c r="F58" t="n">
-        <v>604.3651733398438</v>
+        <v>605.1270751953125</v>
       </c>
       <c r="G58" t="n">
-        <v>603.7385864257812</v>
+        <v>601.6099853515625</v>
       </c>
       <c r="H58" t="n">
         <v>598.6890714285714</v>
@@ -2289,7 +2289,7 @@
         <v>604.9157838555396</v>
       </c>
       <c r="J58" t="n">
-        <v>594.9490966796875</v>
+        <v>595.5479736328125</v>
       </c>
     </row>
     <row r="59">
@@ -2297,7 +2297,7 @@
         <v>643.3404167</v>
       </c>
       <c r="B59" t="n">
-        <v>620.2069702148438</v>
+        <v>620.068603515625</v>
       </c>
       <c r="C59" t="n">
         <v>617.9960492263542</v>
@@ -2309,10 +2309,10 @@
         <v>618.4513570526531</v>
       </c>
       <c r="F59" t="n">
-        <v>604.7637939453125</v>
+        <v>605.524169921875</v>
       </c>
       <c r="G59" t="n">
-        <v>604.204833984375</v>
+        <v>602.0950927734375</v>
       </c>
       <c r="H59" t="n">
         <v>613.7536666714286</v>
@@ -2321,7 +2321,7 @@
         <v>602.5656595901723</v>
       </c>
       <c r="J59" t="n">
-        <v>591.1819458007812</v>
+        <v>591.8998413085938</v>
       </c>
     </row>
     <row r="60">
@@ -2329,7 +2329,7 @@
         <v>775.1095833000001</v>
       </c>
       <c r="B60" t="n">
-        <v>808.133056640625</v>
+        <v>809.3137817382812</v>
       </c>
       <c r="C60" t="n">
         <v>795.31490304052</v>
@@ -2341,10 +2341,10 @@
         <v>811.3535973227424</v>
       </c>
       <c r="F60" t="n">
-        <v>806.5791625976562</v>
+        <v>808.0698852539062</v>
       </c>
       <c r="G60" t="n">
-        <v>823.8644409179688</v>
+        <v>827.12939453125</v>
       </c>
       <c r="H60" t="n">
         <v>801.0423452285713</v>
@@ -2353,7 +2353,7 @@
         <v>720.4146994234502</v>
       </c>
       <c r="J60" t="n">
-        <v>768.4529418945312</v>
+        <v>769.1541748046875</v>
       </c>
     </row>
     <row r="61">
@@ -2361,7 +2361,7 @@
         <v>617.1733333</v>
       </c>
       <c r="B61" t="n">
-        <v>639.1420288085938</v>
+        <v>640.3477783203125</v>
       </c>
       <c r="C61" t="n">
         <v>635.8611801239083</v>
@@ -2373,10 +2373,10 @@
         <v>622.1539712782909</v>
       </c>
       <c r="F61" t="n">
-        <v>625.2022094726562</v>
+        <v>622.0463256835938</v>
       </c>
       <c r="G61" t="n">
-        <v>634.1964721679688</v>
+        <v>642.9488525390625</v>
       </c>
       <c r="H61" t="n">
         <v>661.1299821242856</v>
@@ -2385,7 +2385,7 @@
         <v>628.6528179842625</v>
       </c>
       <c r="J61" t="n">
-        <v>661.195556640625</v>
+        <v>662.8141479492188</v>
       </c>
     </row>
     <row r="62">
@@ -2393,7 +2393,7 @@
         <v>620.6799999999999</v>
       </c>
       <c r="B62" t="n">
-        <v>632.2306518554688</v>
+        <v>633.3775634765625</v>
       </c>
       <c r="C62" t="n">
         <v>628.1617687296668</v>
@@ -2405,10 +2405,10 @@
         <v>618.2751916188178</v>
       </c>
       <c r="F62" t="n">
-        <v>619.2606201171875</v>
+        <v>616.33056640625</v>
       </c>
       <c r="G62" t="n">
-        <v>628.5700073242188</v>
+        <v>636.0687866210938</v>
       </c>
       <c r="H62" t="n">
         <v>654.3560476085712</v>
@@ -2417,7 +2417,7 @@
         <v>624.635908451142</v>
       </c>
       <c r="J62" t="n">
-        <v>629.2527465820312</v>
+        <v>630.15380859375</v>
       </c>
     </row>
     <row r="63">
@@ -2425,7 +2425,7 @@
         <v>637.3004167</v>
       </c>
       <c r="B63" t="n">
-        <v>638.6930541992188</v>
+        <v>639.8948974609375</v>
       </c>
       <c r="C63" t="n">
         <v>635.3612183450616</v>
@@ -2437,10 +2437,10 @@
         <v>621.6515303447819</v>
       </c>
       <c r="F63" t="n">
-        <v>624.8164672851562</v>
+        <v>621.6751708984375</v>
       </c>
       <c r="G63" t="n">
-        <v>633.8310546875</v>
+        <v>642.5021362304688</v>
       </c>
       <c r="H63" t="n">
         <v>658.9747559357141</v>
@@ -2449,7 +2449,7 @@
         <v>627.6841742902054</v>
       </c>
       <c r="J63" t="n">
-        <v>631.0331420898438</v>
+        <v>632.2463989257812</v>
       </c>
     </row>
     <row r="64">
@@ -2457,7 +2457,7 @@
         <v>649.4658333</v>
       </c>
       <c r="B64" t="n">
-        <v>641.5674438476562</v>
+        <v>642.7940063476562</v>
       </c>
       <c r="C64" t="n">
         <v>638.5609737296813</v>
@@ -2469,10 +2469,10 @@
         <v>621.1438408418521</v>
       </c>
       <c r="F64" t="n">
-        <v>627.2857055664062</v>
+        <v>624.0505981445312</v>
       </c>
       <c r="G64" t="n">
-        <v>636.1693725585938</v>
+        <v>645.3613891601562</v>
       </c>
       <c r="H64" t="n">
         <v>668.357559505714</v>
@@ -2481,7 +2481,7 @@
         <v>640.8429835751151</v>
       </c>
       <c r="J64" t="n">
-        <v>646.3473510742188</v>
+        <v>647.3795776367188</v>
       </c>
     </row>
     <row r="65">
@@ -2489,7 +2489,7 @@
         <v>657.14125</v>
       </c>
       <c r="B65" t="n">
-        <v>646.7352905273438</v>
+        <v>648.0068969726562</v>
       </c>
       <c r="C65" t="n">
         <v>644.3105341864202</v>
@@ -2501,10 +2501,10 @@
         <v>626.7003726795106</v>
       </c>
       <c r="F65" t="n">
-        <v>631.7225952148438</v>
+        <v>628.3189086914062</v>
       </c>
       <c r="G65" t="n">
-        <v>640.37109375</v>
+        <v>650.499267578125</v>
       </c>
       <c r="H65" t="n">
         <v>675.2647975999997</v>
@@ -2513,7 +2513,7 @@
         <v>650.3251912506317</v>
       </c>
       <c r="J65" t="n">
-        <v>656.4200439453125</v>
+        <v>657.5159301757812</v>
       </c>
     </row>
     <row r="66">
@@ -2521,7 +2521,7 @@
         <v>657.4141667</v>
       </c>
       <c r="B66" t="n">
-        <v>635.775146484375</v>
+        <v>636.951904296875</v>
       </c>
       <c r="C66" t="n">
         <v>632.111466782557</v>
@@ -2533,10 +2533,10 @@
         <v>621.7490393762246</v>
       </c>
       <c r="F66" t="n">
-        <v>622.3086547851562</v>
+        <v>619.2626953125</v>
       </c>
       <c r="G66" t="n">
-        <v>631.456298828125</v>
+        <v>639.5980834960938</v>
       </c>
       <c r="H66" t="n">
         <v>647.1666309371427</v>
@@ -2545,7 +2545,7 @@
         <v>655.2609033255688</v>
       </c>
       <c r="J66" t="n">
-        <v>660.07373046875</v>
+        <v>660.9413452148438</v>
       </c>
     </row>
     <row r="67">
@@ -2553,7 +2553,7 @@
         <v>642.1116667</v>
       </c>
       <c r="B67" t="n">
-        <v>635.775146484375</v>
+        <v>636.951904296875</v>
       </c>
       <c r="C67" t="n">
         <v>632.111466782557</v>
@@ -2565,10 +2565,10 @@
         <v>621.7490393762246</v>
       </c>
       <c r="F67" t="n">
-        <v>622.3086547851562</v>
+        <v>619.2626953125</v>
       </c>
       <c r="G67" t="n">
-        <v>631.456298828125</v>
+        <v>639.5980834960938</v>
       </c>
       <c r="H67" t="n">
         <v>647.1666309371427</v>
@@ -2577,7 +2577,7 @@
         <v>652.571238601117</v>
       </c>
       <c r="J67" t="n">
-        <v>655.6459350585938</v>
+        <v>656.7798461914062</v>
       </c>
     </row>
     <row r="68">
@@ -2585,7 +2585,7 @@
         <v>649.3841667</v>
       </c>
       <c r="B68" t="n">
-        <v>636.4484252929688</v>
+        <v>637.6309814453125</v>
       </c>
       <c r="C68" t="n">
         <v>632.8614094508273</v>
@@ -2597,10 +2597,10 @@
         <v>622.1378240363582</v>
       </c>
       <c r="F68" t="n">
-        <v>622.8873901367188</v>
+        <v>619.8193969726562</v>
       </c>
       <c r="G68" t="n">
-        <v>632.0042724609375</v>
+        <v>640.2682495117188</v>
       </c>
       <c r="H68" t="n">
         <v>651.8609821271426</v>
@@ -2609,7 +2609,7 @@
         <v>641.5453852651233</v>
       </c>
       <c r="J68" t="n">
-        <v>646.1688842773438</v>
+        <v>647.3544311523438</v>
       </c>
     </row>
     <row r="69">
@@ -2617,7 +2617,7 @@
         <v>647.1404166999999</v>
       </c>
       <c r="B69" t="n">
-        <v>634.0250854492188</v>
+        <v>635.1870727539062</v>
       </c>
       <c r="C69" t="n">
         <v>630.1616158450543</v>
@@ -2629,10 +2629,10 @@
         <v>618.1479231533812</v>
       </c>
       <c r="F69" t="n">
-        <v>620.8038940429688</v>
+        <v>617.815185546875</v>
       </c>
       <c r="G69" t="n">
-        <v>630.0314331054688</v>
+        <v>637.855712890625</v>
       </c>
       <c r="H69" t="n">
         <v>650.9557857028569</v>
@@ -2641,7 +2641,7 @@
         <v>647.6889838755881</v>
       </c>
       <c r="J69" t="n">
-        <v>649.2178344726562</v>
+        <v>650.2532958984375</v>
       </c>
     </row>
     <row r="70">
@@ -2649,7 +2649,7 @@
         <v>658.3666667</v>
       </c>
       <c r="B70" t="n">
-        <v>639.2767333984375</v>
+        <v>640.483642578125</v>
       </c>
       <c r="C70" t="n">
         <v>636.0111686575624</v>
@@ -2661,10 +2661,10 @@
         <v>622.2073385346941</v>
       </c>
       <c r="F70" t="n">
-        <v>625.3179931640625</v>
+        <v>622.1576538085938</v>
       </c>
       <c r="G70" t="n">
-        <v>634.3059692382812</v>
+        <v>643.0828857421875</v>
       </c>
       <c r="H70" t="n">
         <v>661.1299821242856</v>
@@ -2673,7 +2673,7 @@
         <v>645.4837875522602</v>
       </c>
       <c r="J70" t="n">
-        <v>648.9026489257812</v>
+        <v>650.0513916015625</v>
       </c>
     </row>
     <row r="71">
@@ -2681,7 +2681,7 @@
         <v>654.8674999999999</v>
       </c>
       <c r="B71" t="n">
-        <v>637.0318603515625</v>
+        <v>638.2196044921875</v>
       </c>
       <c r="C71" t="n">
         <v>633.5113597633281</v>
@@ -2693,10 +2693,10 @@
         <v>622.1440539237184</v>
       </c>
       <c r="F71" t="n">
-        <v>623.388916015625</v>
+        <v>620.3019409179688</v>
       </c>
       <c r="G71" t="n">
-        <v>632.4793090820312</v>
+        <v>640.84912109375</v>
       </c>
       <c r="H71" t="n">
         <v>651.8609821271426</v>
@@ -2705,7 +2705,7 @@
         <v>656.5869003728088</v>
       </c>
       <c r="J71" t="n">
-        <v>657.0479736328125</v>
+        <v>658.0455932617188</v>
       </c>
     </row>
     <row r="72">
@@ -2713,7 +2713,7 @@
         <v>654.1358332999999</v>
       </c>
       <c r="B72" t="n">
-        <v>639.3216552734375</v>
+        <v>640.5289916992188</v>
       </c>
       <c r="C72" t="n">
         <v>636.061164835447</v>
@@ -2725,10 +2725,10 @@
         <v>622.2073385346941</v>
       </c>
       <c r="F72" t="n">
-        <v>625.3566284179688</v>
+        <v>622.19482421875</v>
       </c>
       <c r="G72" t="n">
-        <v>634.3426513671875</v>
+        <v>643.1275634765625</v>
       </c>
       <c r="H72" t="n">
         <v>661.1299821242856</v>
@@ -2737,7 +2737,7 @@
         <v>653.2026974745862</v>
       </c>
       <c r="J72" t="n">
-        <v>655.0172729492188</v>
+        <v>656.0459594726562</v>
       </c>
     </row>
     <row r="73">
@@ -2745,7 +2745,7 @@
         <v>629.2745833</v>
       </c>
       <c r="B73" t="n">
-        <v>650.3326416015625</v>
+        <v>651.6359252929688</v>
       </c>
       <c r="C73" t="n">
         <v>648.310228417195</v>
@@ -2757,10 +2757,10 @@
         <v>632.3631993541484</v>
       </c>
       <c r="F73" t="n">
-        <v>634.8091430664062</v>
+        <v>631.2880859375</v>
       </c>
       <c r="G73" t="n">
-        <v>643.2939453125</v>
+        <v>654.0733032226562</v>
       </c>
       <c r="H73" t="n">
         <v>666.134904745714</v>
@@ -2769,7 +2769,7 @@
         <v>654.928137841093</v>
       </c>
       <c r="J73" t="n">
-        <v>660.8834228515625</v>
+        <v>661.9308471679688</v>
       </c>
     </row>
     <row r="74">
@@ -2777,7 +2777,7 @@
         <v>629.6404166999999</v>
       </c>
       <c r="B74" t="n">
-        <v>638.6480712890625</v>
+        <v>639.8495483398438</v>
       </c>
       <c r="C74" t="n">
         <v>635.3112221671768</v>
@@ -2789,10 +2789,10 @@
         <v>621.6515303447819</v>
       </c>
       <c r="F74" t="n">
-        <v>624.7778930664062</v>
+        <v>621.6380615234375</v>
       </c>
       <c r="G74" t="n">
-        <v>633.7944946289062</v>
+        <v>642.4573974609375</v>
       </c>
       <c r="H74" t="n">
         <v>658.9747559357141</v>
@@ -2801,7 +2801,7 @@
         <v>634.6167593490011</v>
       </c>
       <c r="J74" t="n">
-        <v>642.8259887695312</v>
+        <v>643.534912109375</v>
       </c>
     </row>
     <row r="75">
@@ -2809,7 +2809,7 @@
         <v>630.6683333</v>
       </c>
       <c r="B75" t="n">
-        <v>631.6476440429688</v>
+        <v>632.7894897460938</v>
       </c>
       <c r="C75" t="n">
         <v>627.5118184171658</v>
@@ -2821,10 +2821,10 @@
         <v>613.9335482539423</v>
       </c>
       <c r="F75" t="n">
-        <v>618.759033203125</v>
+        <v>615.8480224609375</v>
       </c>
       <c r="G75" t="n">
-        <v>628.0950317382812</v>
+        <v>635.488037109375</v>
       </c>
       <c r="H75" t="n">
         <v>654.1528690371425</v>
@@ -2833,7 +2833,7 @@
         <v>630.5726318288362</v>
       </c>
       <c r="J75" t="n">
-        <v>635.3161010742188</v>
+        <v>636.211181640625</v>
       </c>
     </row>
     <row r="76">
@@ -2841,7 +2841,7 @@
         <v>629.8320833</v>
       </c>
       <c r="B76" t="n">
-        <v>630.30224609375</v>
+        <v>631.432861328125</v>
       </c>
       <c r="C76" t="n">
         <v>626.0119330806253</v>
@@ -2853,10 +2853,10 @@
         <v>608.1240329877664</v>
       </c>
       <c r="F76" t="n">
-        <v>617.6016235351562</v>
+        <v>614.7345581054688</v>
       </c>
       <c r="G76" t="n">
-        <v>626.9989013671875</v>
+        <v>634.1475219726562</v>
       </c>
       <c r="H76" t="n">
         <v>649.3340476085712</v>
@@ -2865,7 +2865,7 @@
         <v>625.940136596638</v>
       </c>
       <c r="J76" t="n">
-        <v>636.5519409179688</v>
+        <v>637.6318359375</v>
       </c>
     </row>
     <row r="77">
@@ -2873,7 +2873,7 @@
         <v>637.5841667</v>
       </c>
       <c r="B77" t="n">
-        <v>645.4486083984375</v>
+        <v>646.1837768554688</v>
       </c>
       <c r="C77" t="n">
         <v>636.6250630443385</v>
@@ -2885,10 +2885,10 @@
         <v>609.4456545919152</v>
       </c>
       <c r="F77" t="n">
-        <v>639.7855834960938</v>
+        <v>637.4887084960938</v>
       </c>
       <c r="G77" t="n">
-        <v>640.80419921875</v>
+        <v>641.3377075195312</v>
       </c>
       <c r="H77" t="n">
         <v>641.2656309428569</v>
@@ -2897,7 +2897,7 @@
         <v>628.5948000716255</v>
       </c>
       <c r="J77" t="n">
-        <v>639.3421630859375</v>
+        <v>639.8839111328125</v>
       </c>
     </row>
     <row r="78">
@@ -2905,7 +2905,7 @@
         <v>638.2716667</v>
       </c>
       <c r="B78" t="n">
-        <v>641.3981323242188</v>
+        <v>642.1004028320312</v>
       </c>
       <c r="C78" t="n">
         <v>632.1754032126014</v>
@@ -2917,10 +2917,10 @@
         <v>598.0053390201266</v>
       </c>
       <c r="F78" t="n">
-        <v>636.5335083007812</v>
+        <v>634.3688354492188</v>
       </c>
       <c r="G78" t="n">
-        <v>637.28173828125</v>
+        <v>637.1157836914062</v>
       </c>
       <c r="H78" t="n">
         <v>614.4102380828569</v>
@@ -2929,7 +2929,7 @@
         <v>633.3334418566961</v>
       </c>
       <c r="J78" t="n">
-        <v>635.3126831054688</v>
+        <v>636.4722900390625</v>
       </c>
     </row>
     <row r="79">
@@ -2937,7 +2937,7 @@
         <v>633.75125</v>
       </c>
       <c r="B79" t="n">
-        <v>648.6362915039062</v>
+        <v>649.3975219726562</v>
       </c>
       <c r="C79" t="n">
         <v>640.1247954962664</v>
@@ -2949,10 +2949,10 @@
         <v>617.5412228401129</v>
       </c>
       <c r="F79" t="n">
-        <v>642.343505859375</v>
+        <v>639.942626953125</v>
       </c>
       <c r="G79" t="n">
-        <v>643.5745849609375</v>
+        <v>644.6583251953125</v>
       </c>
       <c r="H79" t="n">
         <v>641.1607380885713</v>
@@ -2961,7 +2961,7 @@
         <v>636.0906102458315</v>
       </c>
       <c r="J79" t="n">
-        <v>636.6021118164062</v>
+        <v>637.9423217773438</v>
       </c>
     </row>
     <row r="80">
@@ -2969,7 +2969,7 @@
         <v>649.3595833000001</v>
       </c>
       <c r="B80" t="n">
-        <v>651.1419067382812</v>
+        <v>651.9237060546875</v>
       </c>
       <c r="C80" t="n">
         <v>642.8745852799243</v>
@@ -2981,10 +2981,10 @@
         <v>618.3499214875046</v>
       </c>
       <c r="F80" t="n">
-        <v>644.3531494140625</v>
+        <v>641.8706665039062</v>
       </c>
       <c r="G80" t="n">
-        <v>645.7513427734375</v>
+        <v>647.2281494140625</v>
       </c>
       <c r="H80" t="n">
         <v>636.8610595142857</v>
@@ -2993,7 +2993,7 @@
         <v>643.6870490860831</v>
       </c>
       <c r="J80" t="n">
-        <v>636.1243286132812</v>
+        <v>637.318359375</v>
       </c>
     </row>
     <row r="81">
@@ -3001,7 +3001,7 @@
         <v>649.6583333</v>
       </c>
       <c r="B81" t="n">
-        <v>646.6324462890625</v>
+        <v>647.3772583007812</v>
       </c>
       <c r="C81" t="n">
         <v>637.9249636693403</v>
@@ -3013,10 +3013,10 @@
         <v>609.2316192689246</v>
       </c>
       <c r="F81" t="n">
-        <v>640.7356567382812</v>
+        <v>638.4002685546875</v>
       </c>
       <c r="G81" t="n">
-        <v>641.8331298828125</v>
+        <v>642.5709838867188</v>
       </c>
       <c r="H81" t="n">
         <v>639.5345952285713</v>
@@ -3025,7 +3025,7 @@
         <v>647.1734455012988</v>
       </c>
       <c r="J81" t="n">
-        <v>643.9988403320312</v>
+        <v>645.0555419921875</v>
       </c>
     </row>
     <row r="82">
@@ -3033,7 +3033,7 @@
         <v>639.0816667</v>
       </c>
       <c r="B82" t="n">
-        <v>642.99072265625</v>
+        <v>643.7059936523438</v>
       </c>
       <c r="C82" t="n">
         <v>633.9252694385655</v>
@@ -3045,10 +3045,10 @@
         <v>604.2917117587099</v>
       </c>
       <c r="F82" t="n">
-        <v>637.8124389648438</v>
+        <v>635.5957641601562</v>
       </c>
       <c r="G82" t="n">
-        <v>638.6670532226562</v>
+        <v>638.7760620117188</v>
       </c>
       <c r="H82" t="n">
         <v>614.8440595142856</v>
@@ -3057,7 +3057,7 @@
         <v>641.7764987110194</v>
       </c>
       <c r="J82" t="n">
-        <v>643.2783203125</v>
+        <v>644.452392578125</v>
       </c>
     </row>
     <row r="83">
@@ -3065,7 +3065,7 @@
         <v>638.1045832999999</v>
       </c>
       <c r="B83" t="n">
-        <v>645.7218017578125</v>
+        <v>646.4591674804688</v>
       </c>
       <c r="C83" t="n">
         <v>636.9250401116467</v>
@@ -3077,10 +3077,10 @@
         <v>609.0926344311486</v>
       </c>
       <c r="F83" t="n">
-        <v>640.0048828125</v>
+        <v>637.6990966796875</v>
       </c>
       <c r="G83" t="n">
-        <v>641.041748046875</v>
+        <v>641.6223754882812</v>
       </c>
       <c r="H83" t="n">
         <v>641.2656309428569</v>
@@ -3089,7 +3089,7 @@
         <v>631.596765360038</v>
       </c>
       <c r="J83" t="n">
-        <v>635.0538940429688</v>
+        <v>636.3738403320312</v>
       </c>
     </row>
     <row r="84">
@@ -3097,7 +3097,7 @@
         <v>651.2941667</v>
       </c>
       <c r="B84" t="n">
-        <v>653.1013793945312</v>
+        <v>653.8995361328125</v>
       </c>
       <c r="C84" t="n">
         <v>645.0244209289657</v>
@@ -3109,10 +3109,10 @@
         <v>620.9940450521668</v>
       </c>
       <c r="F84" t="n">
-        <v>645.9244995117188</v>
+        <v>643.3779907226562</v>
       </c>
       <c r="G84" t="n">
-        <v>647.4532470703125</v>
+        <v>649.2271118164062</v>
       </c>
       <c r="H84" t="n">
         <v>637.3927202271427</v>
@@ -3121,7 +3121,7 @@
         <v>639.645009996139</v>
       </c>
       <c r="J84" t="n">
-        <v>637.5048217773438</v>
+        <v>638.8206787109375</v>
       </c>
     </row>
     <row r="85">
@@ -3129,7 +3129,7 @@
         <v>645.9495833</v>
       </c>
       <c r="B85" t="n">
-        <v>645.5852661132812</v>
+        <v>646.3214721679688</v>
       </c>
       <c r="C85" t="n">
         <v>636.7750515779926</v>
@@ -3141,10 +3141,10 @@
         <v>609.0926344311486</v>
       </c>
       <c r="F85" t="n">
-        <v>639.895263671875</v>
+        <v>637.5939331054688</v>
       </c>
       <c r="G85" t="n">
-        <v>640.9229125976562</v>
+        <v>641.47998046875</v>
       </c>
       <c r="H85" t="n">
         <v>641.2656309428569</v>
@@ -3153,7 +3153,7 @@
         <v>647.3791788649077</v>
       </c>
       <c r="J85" t="n">
-        <v>647.7022094726562</v>
+        <v>648.7015991210938</v>
       </c>
     </row>
     <row r="86">
@@ -3161,7 +3161,7 @@
         <v>652.5133333</v>
       </c>
       <c r="B86" t="n">
-        <v>644.5380859375</v>
+        <v>645.2658081054688</v>
       </c>
       <c r="C86" t="n">
         <v>635.6251394866447</v>
@@ -3173,10 +3173,10 @@
         <v>608.942449557821</v>
       </c>
       <c r="F86" t="n">
-        <v>639.0548095703125</v>
+        <v>636.7876586914062</v>
       </c>
       <c r="G86" t="n">
-        <v>640.0127563476562</v>
+        <v>640.3890380859375</v>
       </c>
       <c r="H86" t="n">
         <v>636.1052499885712</v>
@@ -3185,7 +3185,7 @@
         <v>642.4113944825885</v>
       </c>
       <c r="J86" t="n">
-        <v>641.650146484375</v>
+        <v>642.84814453125</v>
       </c>
     </row>
     <row r="87">
@@ -3193,7 +3193,7 @@
         <v>653.145</v>
       </c>
       <c r="B87" t="n">
-        <v>636.4862060546875</v>
+        <v>637.1492919921875</v>
       </c>
       <c r="C87" t="n">
         <v>626.7758160010553</v>
@@ -3205,10 +3205,10 @@
         <v>594.321418165349</v>
       </c>
       <c r="F87" t="n">
-        <v>632.5870971679688</v>
+        <v>630.5828247070312</v>
       </c>
       <c r="G87" t="n">
-        <v>633.007568359375</v>
+        <v>631.9970092773438</v>
       </c>
       <c r="H87" t="n">
         <v>600.5466904628571</v>
@@ -3217,7 +3217,7 @@
         <v>641.9983348242614</v>
       </c>
       <c r="J87" t="n">
-        <v>642.1072387695312</v>
+        <v>643.3162841796875</v>
       </c>
     </row>
     <row r="88">
@@ -3225,7 +3225,7 @@
         <v>654.24375</v>
       </c>
       <c r="B88" t="n">
-        <v>662.9069213867188</v>
+        <v>663.7874755859375</v>
       </c>
       <c r="C88" t="n">
         <v>655.7735991741731</v>
@@ -3237,10 +3237,10 @@
         <v>622.6461832047383</v>
       </c>
       <c r="F88" t="n">
-        <v>654.298583984375</v>
+        <v>651.8026733398438</v>
       </c>
       <c r="G88" t="n">
-        <v>655.9623413085938</v>
+        <v>659.2218017578125</v>
       </c>
       <c r="H88" t="n">
         <v>649.5104404599999</v>
@@ -3249,7 +3249,7 @@
         <v>649.8375026940342</v>
       </c>
       <c r="J88" t="n">
-        <v>648.64404296875</v>
+        <v>650.3270874023438</v>
       </c>
     </row>
     <row r="89">
@@ -3257,7 +3257,7 @@
         <v>657.9450000000001</v>
       </c>
       <c r="B89" t="n">
-        <v>678.6650390625</v>
+        <v>679.6821899414062</v>
       </c>
       <c r="C89" t="n">
         <v>673.0222805443898</v>
@@ -3269,10 +3269,10 @@
         <v>640.8279416720409</v>
       </c>
       <c r="F89" t="n">
-        <v>669.8079223632812</v>
+        <v>666.8141479492188</v>
       </c>
       <c r="G89" t="n">
-        <v>669.6163940429688</v>
+        <v>675.2598876953125</v>
       </c>
       <c r="H89" t="n">
         <v>671.932047602857</v>
@@ -3281,7 +3281,7 @@
         <v>666.6145196464745</v>
       </c>
       <c r="J89" t="n">
-        <v>667.0198974609375</v>
+        <v>668.2750854492188</v>
       </c>
     </row>
     <row r="90">
@@ -3289,7 +3289,7 @@
         <v>656.8808332999999</v>
       </c>
       <c r="B90" t="n">
-        <v>678.0250854492188</v>
+        <v>679.03662109375</v>
       </c>
       <c r="C90" t="n">
         <v>672.3223340540042</v>
@@ -3301,10 +3301,10 @@
         <v>639.6665670615298</v>
       </c>
       <c r="F90" t="n">
-        <v>669.1785278320312</v>
+        <v>666.2050170898438</v>
       </c>
       <c r="G90" t="n">
-        <v>669.062255859375</v>
+        <v>674.6090087890625</v>
       </c>
       <c r="H90" t="n">
         <v>658.3798571257141</v>
@@ -3313,7 +3313,7 @@
         <v>670.7447532560813</v>
       </c>
       <c r="J90" t="n">
-        <v>674.4236450195312</v>
+        <v>675.283935546875</v>
       </c>
     </row>
     <row r="91">
@@ -3321,7 +3321,7 @@
         <v>662.5716667</v>
       </c>
       <c r="B91" t="n">
-        <v>667.6544189453125</v>
+        <v>668.5755004882812</v>
       </c>
       <c r="C91" t="n">
         <v>660.9732016741805</v>
@@ -3333,10 +3333,10 @@
         <v>629.2662345725886</v>
       </c>
       <c r="F91" t="n">
-        <v>658.9737548828125</v>
+        <v>656.327880859375</v>
       </c>
       <c r="G91" t="n">
-        <v>660.0782470703125</v>
+        <v>664.0565185546875</v>
       </c>
       <c r="H91" t="n">
         <v>645.293547602857</v>
@@ -3345,7 +3345,7 @@
         <v>667.8925772138724</v>
       </c>
       <c r="J91" t="n">
-        <v>669.4423828125</v>
+        <v>670.2678833007812</v>
       </c>
     </row>
     <row r="92">
@@ -3353,7 +3353,7 @@
         <v>661.8104167</v>
       </c>
       <c r="B92" t="n">
-        <v>643.3092041015625</v>
+        <v>644.0270385742188</v>
       </c>
       <c r="C92" t="n">
         <v>634.2752426837583</v>
@@ -3365,10 +3365,10 @@
         <v>604.8889418680529</v>
       </c>
       <c r="F92" t="n">
-        <v>638.0682373046875</v>
+        <v>635.8411254882812</v>
       </c>
       <c r="G92" t="n">
-        <v>638.944091796875</v>
+        <v>639.1083374023438</v>
       </c>
       <c r="H92" t="n">
         <v>616.3047738028571</v>
@@ -3377,7 +3377,7 @@
         <v>667.2720517613288</v>
       </c>
       <c r="J92" t="n">
-        <v>659.9166870117188</v>
+        <v>660.7671508789062</v>
       </c>
     </row>
     <row r="93">
@@ -3385,7 +3385,7 @@
         <v>653.7116667</v>
       </c>
       <c r="B93" t="n">
-        <v>641.3524780273438</v>
+        <v>642.0546264648438</v>
       </c>
       <c r="C93" t="n">
         <v>632.1254070347168</v>
@@ -3397,10 +3397,10 @@
         <v>598.0053390201266</v>
       </c>
       <c r="F93" t="n">
-        <v>636.4969482421875</v>
+        <v>634.333740234375</v>
       </c>
       <c r="G93" t="n">
-        <v>637.2423706054688</v>
+        <v>637.0684204101562</v>
       </c>
       <c r="H93" t="n">
         <v>614.4102380828569</v>
@@ -3409,7 +3409,7 @@
         <v>649.8284355745163</v>
       </c>
       <c r="J93" t="n">
-        <v>648.7593383789062</v>
+        <v>650.0707397460938</v>
       </c>
     </row>
     <row r="94">
@@ -3417,7 +3417,7 @@
         <v>645.9745832999999</v>
       </c>
       <c r="B94" t="n">
-        <v>643.5368041992188</v>
+        <v>644.25634765625</v>
       </c>
       <c r="C94" t="n">
         <v>634.5252235731816</v>
@@ -3429,10 +3429,10 @@
         <v>604.8889418680529</v>
       </c>
       <c r="F94" t="n">
-        <v>638.2508544921875</v>
+        <v>636.0164184570312</v>
       </c>
       <c r="G94" t="n">
-        <v>639.1420288085938</v>
+        <v>639.3453369140625</v>
       </c>
       <c r="H94" t="n">
         <v>617.8801071371429</v>
@@ -3441,7 +3441,7 @@
         <v>647.745948557982</v>
       </c>
       <c r="J94" t="n">
-        <v>643.974609375</v>
+        <v>645.283935546875</v>
       </c>
     </row>
     <row r="95">
@@ -3449,7 +3449,7 @@
         <v>657.925</v>
       </c>
       <c r="B95" t="n">
-        <v>643.67333984375</v>
+        <v>644.3941040039062</v>
       </c>
       <c r="C95" t="n">
         <v>634.6752121068357</v>
@@ -3461,10 +3461,10 @@
         <v>605.0558070424531</v>
       </c>
       <c r="F95" t="n">
-        <v>638.3605346679688</v>
+        <v>636.12158203125</v>
       </c>
       <c r="G95" t="n">
-        <v>639.2607421875</v>
+        <v>639.48779296875</v>
       </c>
       <c r="H95" t="n">
         <v>619.7978690428571</v>
@@ -3473,7 +3473,7 @@
         <v>643.1242566426707</v>
       </c>
       <c r="J95" t="n">
-        <v>640.6458740234375</v>
+        <v>641.8037719726562</v>
       </c>
     </row>
     <row r="96">
@@ -3481,7 +3481,7 @@
         <v>657.4579167000001</v>
       </c>
       <c r="B96" t="n">
-        <v>642.3079833984375</v>
+        <v>643.0177001953125</v>
       </c>
       <c r="C96" t="n">
         <v>633.1753267702952</v>
@@ -3493,10 +3493,10 @@
         <v>603.6740635119571</v>
       </c>
       <c r="F96" t="n">
-        <v>637.2642822265625</v>
+        <v>635.0698852539062</v>
       </c>
       <c r="G96" t="n">
-        <v>638.0733642578125</v>
+        <v>638.0646362304688</v>
       </c>
       <c r="H96" t="n">
         <v>615.0564880857142</v>
@@ -3505,7 +3505,7 @@
         <v>649.5425237922527</v>
       </c>
       <c r="J96" t="n">
-        <v>646.9374389648438</v>
+        <v>648.14404296875</v>
       </c>
     </row>
     <row r="97">
@@ -3513,7 +3513,7 @@
         <v>645.5066667</v>
       </c>
       <c r="B97" t="n">
-        <v>640.9431762695312</v>
+        <v>641.641845703125</v>
       </c>
       <c r="C97" t="n">
         <v>631.6754414337545</v>
@@ -3525,10 +3525,10 @@
         <v>598.8774410435901</v>
       </c>
       <c r="F97" t="n">
-        <v>636.1680908203125</v>
+        <v>634.0182495117188</v>
       </c>
       <c r="G97" t="n">
-        <v>636.8861083984375</v>
+        <v>636.6414794921875</v>
       </c>
       <c r="H97" t="n">
         <v>617.165535702857</v>
@@ -3537,7 +3537,7 @@
         <v>647.1690735940998</v>
       </c>
       <c r="J97" t="n">
-        <v>645.8168334960938</v>
+        <v>646.97265625</v>
       </c>
     </row>
     <row r="98">
@@ -3545,7 +3545,7 @@
         <v>659.9454167</v>
       </c>
       <c r="B98" t="n">
-        <v>663.2265625</v>
+        <v>664.109619140625</v>
       </c>
       <c r="C98" t="n">
         <v>656.1235724193659</v>
@@ -3557,10 +3557,10 @@
         <v>624.3341194582606</v>
       </c>
       <c r="F98" t="n">
-        <v>654.6132202148438</v>
+        <v>652.1072387695312</v>
       </c>
       <c r="G98" t="n">
-        <v>656.2392578125</v>
+        <v>659.5472412109375</v>
       </c>
       <c r="H98" t="n">
         <v>661.5000476028571</v>
@@ -3569,7 +3569,7 @@
         <v>648.6005470747758</v>
       </c>
       <c r="J98" t="n">
-        <v>644.9419555664062</v>
+        <v>646.3535766601562</v>
       </c>
     </row>
     <row r="99">
@@ -3577,7 +3577,7 @@
         <v>649.0525</v>
       </c>
       <c r="B99" t="n">
-        <v>673.8206176757812</v>
+        <v>674.7952880859375</v>
       </c>
       <c r="C99" t="n">
         <v>667.722685688613</v>
@@ -3589,10 +3589,10 @@
         <v>633.9086273143387</v>
       </c>
       <c r="F99" t="n">
-        <v>665.0426635742188</v>
+        <v>662.2019653320312</v>
       </c>
       <c r="G99" t="n">
-        <v>665.4212646484375</v>
+        <v>670.332275390625</v>
       </c>
       <c r="H99" t="n">
         <v>649.7823333171428</v>
@@ -3601,7 +3601,7 @@
         <v>674.4820210728376</v>
       </c>
       <c r="J99" t="n">
-        <v>668.353515625</v>
+        <v>669.43115234375</v>
       </c>
     </row>
     <row r="100">
@@ -3609,7 +3609,7 @@
         <v>658.20125</v>
       </c>
       <c r="B100" t="n">
-        <v>664.093505859375</v>
+        <v>664.9841918945312</v>
       </c>
       <c r="C100" t="n">
         <v>657.0734997991749</v>
@@ -3621,10 +3621,10 @@
         <v>625.4259066638075</v>
       </c>
       <c r="F100" t="n">
-        <v>655.46728515625</v>
+        <v>652.9339599609375</v>
       </c>
       <c r="G100" t="n">
-        <v>656.9912109375</v>
+        <v>660.4303588867188</v>
       </c>
       <c r="H100" t="n">
         <v>655.8860833171427</v>
@@ -3633,7 +3633,7 @@
         <v>658.610479518701</v>
       </c>
       <c r="J100" t="n">
-        <v>663.0299682617188</v>
+        <v>663.7188110351562</v>
       </c>
     </row>
     <row r="101">
@@ -3641,7 +3641,7 @@
         <v>667.5704167</v>
       </c>
       <c r="B101" t="n">
-        <v>648.8639526367188</v>
+        <v>649.6271362304688</v>
       </c>
       <c r="C101" t="n">
         <v>640.37477638569</v>
@@ -3653,10 +3653,10 @@
         <v>618.071734409968</v>
       </c>
       <c r="F101" t="n">
-        <v>642.526123046875</v>
+        <v>640.117919921875</v>
       </c>
       <c r="G101" t="n">
-        <v>643.7725830078125</v>
+        <v>644.8953857421875</v>
       </c>
       <c r="H101" t="n">
         <v>639.7000952314283</v>
@@ -3665,7 +3665,7 @@
         <v>664.7429506535831</v>
       </c>
       <c r="J101" t="n">
-        <v>660.14208984375</v>
+        <v>660.9747314453125</v>
       </c>
     </row>
     <row r="102">
@@ -3673,7 +3673,7 @@
         <v>668.5225</v>
       </c>
       <c r="B102" t="n">
-        <v>649.501708984375</v>
+        <v>650.27001953125</v>
       </c>
       <c r="C102" t="n">
         <v>641.0747228760756</v>
@@ -3685,10 +3685,10 @@
         <v>616.2575049903088</v>
       </c>
       <c r="F102" t="n">
-        <v>643.0377807617188</v>
+        <v>640.6087036132812</v>
       </c>
       <c r="G102" t="n">
-        <v>644.3265991210938</v>
+        <v>645.5546264648438</v>
       </c>
       <c r="H102" t="n">
         <v>641.8315357085713</v>
@@ -3697,7 +3697,7 @@
         <v>679.2772506578217</v>
       </c>
       <c r="J102" t="n">
-        <v>659.283447265625</v>
+        <v>660.5167236328125</v>
       </c>
     </row>
     <row r="103">
@@ -3705,7 +3705,7 @@
         <v>650.7575000000001</v>
       </c>
       <c r="B103" t="n">
-        <v>654.4688110351562</v>
+        <v>655.2783203125</v>
       </c>
       <c r="C103" t="n">
         <v>646.5243062655063</v>
@@ -3717,10 +3717,10 @@
         <v>617.7651155852489</v>
       </c>
       <c r="F103" t="n">
-        <v>647.0206298828125</v>
+        <v>644.4296875</v>
       </c>
       <c r="G103" t="n">
-        <v>648.6405639648438</v>
+        <v>650.621826171875</v>
       </c>
       <c r="H103" t="n">
         <v>643.8397678442857</v>
@@ -3729,7 +3729,7 @@
         <v>681.4683015029765</v>
       </c>
       <c r="J103" t="n">
-        <v>661.1940307617188</v>
+        <v>662.4231567382812</v>
       </c>
     </row>
     <row r="104">
@@ -3737,7 +3737,7 @@
         <v>657.9416667</v>
       </c>
       <c r="B104" t="n">
-        <v>659.3482055664062</v>
+        <v>660.1986083984375</v>
       </c>
       <c r="C104" t="n">
         <v>651.8738972991677</v>
@@ -3749,10 +3749,10 @@
         <v>619.2775627164344</v>
       </c>
       <c r="F104" t="n">
-        <v>650.9305419921875</v>
+        <v>648.4087524414062</v>
       </c>
       <c r="G104" t="n">
-        <v>652.8751831054688</v>
+        <v>655.5958862304688</v>
       </c>
       <c r="H104" t="n">
         <v>665.5082023657142</v>
@@ -3761,7 +3761,7 @@
         <v>661.2590098945877</v>
       </c>
       <c r="J104" t="n">
-        <v>654.8388671875</v>
+        <v>655.9332275390625</v>
       </c>
     </row>
     <row r="105">
@@ -3769,7 +3769,7 @@
         <v>659.2345833000001</v>
       </c>
       <c r="B105" t="n">
-        <v>668.567626953125</v>
+        <v>669.4966430664062</v>
       </c>
       <c r="C105" t="n">
         <v>661.9731252318742</v>
@@ -3781,10 +3781,10 @@
         <v>630.045070948491</v>
       </c>
       <c r="F105" t="n">
-        <v>659.8728637695312</v>
+        <v>657.1981201171875</v>
       </c>
       <c r="G105" t="n">
-        <v>660.8699340820312</v>
+        <v>664.986083984375</v>
       </c>
       <c r="H105" t="n">
         <v>645.293547602857</v>
@@ -3793,7 +3793,7 @@
         <v>672.8595600732727</v>
       </c>
       <c r="J105" t="n">
-        <v>665.543212890625</v>
+        <v>666.73828125</v>
       </c>
     </row>
     <row r="106">
@@ -3801,7 +3801,7 @@
         <v>659.05875</v>
       </c>
       <c r="B106" t="n">
-        <v>668.658935546875</v>
+        <v>669.5888671875</v>
       </c>
       <c r="C106" t="n">
         <v>662.0731175876435</v>
@@ -3813,10 +3813,10 @@
         <v>630.045070948491</v>
       </c>
       <c r="F106" t="n">
-        <v>659.9628295898438</v>
+        <v>657.2850952148438</v>
       </c>
       <c r="G106" t="n">
-        <v>660.948974609375</v>
+        <v>665.0791625976562</v>
       </c>
       <c r="H106" t="n">
         <v>645.293547602857</v>
@@ -3825,7 +3825,7 @@
         <v>678.9310908443912</v>
       </c>
       <c r="J106" t="n">
-        <v>669.1276245117188</v>
+        <v>670.1701049804688</v>
       </c>
     </row>
     <row r="107">
@@ -3833,7 +3833,7 @@
         <v>658.5229167</v>
       </c>
       <c r="B107" t="n">
-        <v>686.2099609375</v>
+        <v>687.29443359375</v>
       </c>
       <c r="C107" t="n">
         <v>681.2716498953629</v>
@@ -3845,10 +3845,10 @@
         <v>642.124313577666</v>
       </c>
       <c r="F107" t="n">
-        <v>673.9814453125</v>
+        <v>671.7078247070312</v>
       </c>
       <c r="G107" t="n">
-        <v>676.1466064453125</v>
+        <v>682.9302368164062</v>
       </c>
       <c r="H107" t="n">
         <v>670.3808571171427</v>
@@ -3857,7 +3857,7 @@
         <v>680.5177045243928</v>
       </c>
       <c r="J107" t="n">
-        <v>676.1849975585938</v>
+        <v>677.5267333984375</v>
       </c>
     </row>
     <row r="108">
@@ -3865,7 +3865,7 @@
         <v>596.4270833</v>
       </c>
       <c r="B108" t="n">
-        <v>710.596923828125</v>
+        <v>711.8460693359375</v>
       </c>
       <c r="C108" t="n">
         <v>702.8995195236091</v>
@@ -3877,10 +3877,10 @@
         <v>644.6650236906629</v>
       </c>
       <c r="F108" t="n">
-        <v>672.5480346679688</v>
+        <v>668.9588012695312</v>
       </c>
       <c r="G108" t="n">
-        <v>702.5918579101562</v>
+        <v>708.3751831054688</v>
       </c>
       <c r="H108" t="n">
         <v>673.8018928542856</v>
@@ -3889,7 +3889,7 @@
         <v>661.3297896995134</v>
       </c>
       <c r="J108" t="n">
-        <v>690.7241821289062</v>
+        <v>690.7757568359375</v>
       </c>
     </row>
     <row r="109">
@@ -3897,7 +3897,7 @@
         <v>655.4458333</v>
       </c>
       <c r="B109" t="n">
-        <v>703.4505615234375</v>
+        <v>704.63623046875</v>
       </c>
       <c r="C109" t="n">
         <v>695.2501043072523</v>
@@ -3909,10 +3909,10 @@
         <v>644.4122804909047</v>
       </c>
       <c r="F109" t="n">
-        <v>669.2205200195312</v>
+        <v>666.07568359375</v>
       </c>
       <c r="G109" t="n">
-        <v>696.552734375</v>
+        <v>700.6730346679688</v>
       </c>
       <c r="H109" t="n">
         <v>675.2709999971428</v>
@@ -3921,7 +3921,7 @@
         <v>622.9019307792636</v>
       </c>
       <c r="J109" t="n">
-        <v>648.0767211914062</v>
+        <v>648.5962524414062</v>
       </c>
     </row>
     <row r="110">
@@ -3929,7 +3929,7 @@
         <v>659.2925</v>
       </c>
       <c r="B110" t="n">
-        <v>700.7889404296875</v>
+        <v>701.9511108398438</v>
       </c>
       <c r="C110" t="n">
         <v>692.4003221678252</v>
@@ -3941,10 +3941,10 @@
         <v>645.7513867055983</v>
       </c>
       <c r="F110" t="n">
-        <v>667.98095703125</v>
+        <v>665.0015869140625</v>
       </c>
       <c r="G110" t="n">
-        <v>694.302978515625</v>
+        <v>697.8035278320312</v>
       </c>
       <c r="H110" t="n">
         <v>675.2709999971428</v>
@@ -3953,7 +3953,7 @@
         <v>665.4200778924597</v>
       </c>
       <c r="J110" t="n">
-        <v>681.22802734375</v>
+        <v>681.8360595703125</v>
       </c>
     </row>
     <row r="111">
@@ -3961,7 +3961,7 @@
         <v>657.4</v>
       </c>
       <c r="B111" t="n">
-        <v>685.7620849609375</v>
+        <v>686.7948608398438</v>
       </c>
       <c r="C111" t="n">
         <v>676.3015528889564</v>
@@ -3973,10 +3973,10 @@
         <v>636.464041116368</v>
       </c>
       <c r="F111" t="n">
-        <v>660.9782104492188</v>
+        <v>658.9338989257812</v>
       </c>
       <c r="G111" t="n">
-        <v>681.5930786132812</v>
+        <v>681.593505859375</v>
       </c>
       <c r="H111" t="n">
         <v>658.0589642685713</v>
@@ -3985,7 +3985,7 @@
         <v>674.2919932348148</v>
       </c>
       <c r="J111" t="n">
-        <v>677.1014404296875</v>
+        <v>677.6016845703125</v>
       </c>
     </row>
     <row r="112">
@@ -3993,7 +3993,7 @@
         <v>654.7895833</v>
       </c>
       <c r="B112" t="n">
-        <v>712.9329223632812</v>
+        <v>714.2029418945312</v>
       </c>
       <c r="C112" t="n">
         <v>705.3993284178434</v>
@@ -4005,10 +4005,10 @@
         <v>644.7064206549709</v>
       </c>
       <c r="F112" t="n">
-        <v>673.6353149414062</v>
+        <v>669.9009399414062</v>
       </c>
       <c r="G112" t="n">
-        <v>704.5654296875</v>
+        <v>710.8922729492188</v>
       </c>
       <c r="H112" t="n">
         <v>673.6528928542855</v>
@@ -4017,7 +4017,7 @@
         <v>666.4980901237772</v>
       </c>
       <c r="J112" t="n">
-        <v>680.4561767578125</v>
+        <v>681.6091918945312</v>
       </c>
     </row>
     <row r="113">
@@ -4025,7 +4025,7 @@
         <v>658.19375</v>
       </c>
       <c r="B113" t="n">
-        <v>709.1488037109375</v>
+        <v>710.3849487304688</v>
       </c>
       <c r="C113" t="n">
         <v>701.3496380091839</v>
@@ -4037,10 +4037,10 @@
         <v>644.6650236906629</v>
       </c>
       <c r="F113" t="n">
-        <v>671.873779296875</v>
+        <v>668.3745727539062</v>
       </c>
       <c r="G113" t="n">
-        <v>701.3683471679688</v>
+        <v>706.8146362304688</v>
       </c>
       <c r="H113" t="n">
         <v>673.8018928542856</v>
@@ -4049,7 +4049,7 @@
         <v>663.8352802792588</v>
       </c>
       <c r="J113" t="n">
-        <v>686.7233276367188</v>
+        <v>687.1241455078125</v>
       </c>
     </row>
     <row r="114">
@@ -4057,7 +4057,7 @@
         <v>657.48125</v>
       </c>
       <c r="B114" t="n">
-        <v>702.4232177734375</v>
+        <v>703.599853515625</v>
       </c>
       <c r="C114" t="n">
         <v>694.1501883937892</v>
@@ -4069,10 +4069,10 @@
         <v>644.4122804909047</v>
       </c>
       <c r="F114" t="n">
-        <v>668.7421264648438</v>
+        <v>665.6611938476562</v>
       </c>
       <c r="G114" t="n">
-        <v>695.684326171875</v>
+        <v>699.5654907226562</v>
       </c>
       <c r="H114" t="n">
         <v>675.2709999971428</v>
@@ -4081,7 +4081,7 @@
         <v>669.6290258780148</v>
       </c>
       <c r="J114" t="n">
-        <v>685.14990234375</v>
+        <v>685.582763671875</v>
       </c>
     </row>
     <row r="115">
@@ -4089,7 +4089,7 @@
         <v>656.00125</v>
       </c>
       <c r="B115" t="n">
-        <v>706.7665405273438</v>
+        <v>707.9814453125</v>
       </c>
       <c r="C115" t="n">
         <v>698.7998329370648</v>
@@ -4101,10 +4101,10 @@
         <v>644.6229790520765</v>
       </c>
       <c r="F115" t="n">
-        <v>670.7646484375</v>
+        <v>667.4136352539062</v>
       </c>
       <c r="G115" t="n">
-        <v>699.3552856445312</v>
+        <v>704.2471923828125</v>
       </c>
       <c r="H115" t="n">
         <v>673.6601071399999</v>
@@ -4113,7 +4113,7 @@
         <v>668.7140473806252</v>
       </c>
       <c r="J115" t="n">
-        <v>683.825927734375</v>
+        <v>684.4570922851562</v>
       </c>
     </row>
     <row r="116">
@@ -4121,7 +4121,7 @@
         <v>657.85375</v>
       </c>
       <c r="B116" t="n">
-        <v>697.5674438476562</v>
+        <v>698.7017211914062</v>
       </c>
       <c r="C116" t="n">
         <v>688.9505858937819</v>
@@ -4133,10 +4133,10 @@
         <v>644.4807939599481</v>
       </c>
       <c r="F116" t="n">
-        <v>666.4804077148438</v>
+        <v>663.7013549804688</v>
       </c>
       <c r="G116" t="n">
-        <v>691.5792846679688</v>
+        <v>694.3300170898438</v>
       </c>
       <c r="H116" t="n">
         <v>679.1680952142856</v>
@@ -4145,7 +4145,7 @@
         <v>665.4310215657653</v>
       </c>
       <c r="J116" t="n">
-        <v>681.026611328125</v>
+        <v>681.4545288085938</v>
       </c>
     </row>
     <row r="117">
@@ -4153,7 +4153,7 @@
         <v>654.1308332999999</v>
       </c>
       <c r="B117" t="n">
-        <v>695.8870239257812</v>
+        <v>697.006591796875</v>
       </c>
       <c r="C117" t="n">
         <v>687.1507234899332</v>
@@ -4165,10 +4165,10 @@
         <v>643.6324374634896</v>
       </c>
       <c r="F117" t="n">
-        <v>665.697509765625</v>
+        <v>663.0230102539062</v>
       </c>
       <c r="G117" t="n">
-        <v>690.1583862304688</v>
+        <v>692.5176391601562</v>
       </c>
       <c r="H117" t="n">
         <v>680.0520118799998</v>
@@ -4177,7 +4177,7 @@
         <v>667.2766029310062</v>
       </c>
       <c r="J117" t="n">
-        <v>677.7852783203125</v>
+        <v>678.38037109375</v>
       </c>
     </row>
     <row r="118">
@@ -4185,7 +4185,7 @@
         <v>461.9275</v>
       </c>
       <c r="B118" t="n">
-        <v>497.3310241699219</v>
+        <v>496.7421875</v>
       </c>
       <c r="C118" t="n">
         <v>514.0131578540811</v>
@@ -4197,10 +4197,10 @@
         <v>472.4596215685293</v>
       </c>
       <c r="F118" t="n">
-        <v>467.2945861816406</v>
+        <v>466.3118591308594</v>
       </c>
       <c r="G118" t="n">
-        <v>496.3995971679688</v>
+        <v>488.7505493164062</v>
       </c>
       <c r="H118" t="n">
         <v>474.9925714285714</v>
@@ -4209,7 +4209,7 @@
         <v>574.1085644966338</v>
       </c>
       <c r="J118" t="n">
-        <v>495.9192810058594</v>
+        <v>495.0864868164062</v>
       </c>
     </row>
     <row r="119">
@@ -4217,7 +4217,7 @@
         <v>457.835</v>
       </c>
       <c r="B119" t="n">
-        <v>498.4555358886719</v>
+        <v>497.8722534179688</v>
       </c>
       <c r="C119" t="n">
         <v>515.3630546569676</v>
@@ -4229,10 +4229,10 @@
         <v>473.1011750536756</v>
       </c>
       <c r="F119" t="n">
-        <v>467.6545715332031</v>
+        <v>466.59228515625</v>
       </c>
       <c r="G119" t="n">
-        <v>497.0147094726562</v>
+        <v>489.3920288085938</v>
       </c>
       <c r="H119" t="n">
         <v>474.9925714285714</v>
@@ -4241,7 +4241,7 @@
         <v>470.8221614185427</v>
       </c>
       <c r="J119" t="n">
-        <v>469.3854064941406</v>
+        <v>469.4503173828125</v>
       </c>
     </row>
     <row r="120">
@@ -4249,7 +4249,7 @@
         <v>460.98</v>
       </c>
       <c r="B120" t="n">
-        <v>496.4981384277344</v>
+        <v>495.9052734375</v>
       </c>
       <c r="C120" t="n">
         <v>513.0132342963874</v>
@@ -4261,10 +4261,10 @@
         <v>472.4596215685293</v>
       </c>
       <c r="F120" t="n">
-        <v>467.0279541015625</v>
+        <v>466.1040954589844</v>
       </c>
       <c r="G120" t="n">
-        <v>495.9439697265625</v>
+        <v>488.2752380371094</v>
       </c>
       <c r="H120" t="n">
         <v>474.9925714285714</v>
@@ -4273,7 +4273,7 @@
         <v>467.9061584251655</v>
       </c>
       <c r="J120" t="n">
-        <v>467.9105224609375</v>
+        <v>468.0050354003906</v>
       </c>
     </row>
     <row r="121">
@@ -4281,7 +4281,7 @@
         <v>573.2504167</v>
       </c>
       <c r="B121" t="n">
-        <v>695.6679077148438</v>
+        <v>695.3314208984375</v>
       </c>
       <c r="C121" t="n">
         <v>689.5893483578147</v>
@@ -4293,10 +4293,10 @@
         <v>593.7462804307006</v>
       </c>
       <c r="F121" t="n">
-        <v>562.858642578125</v>
+        <v>547.0657348632812</v>
       </c>
       <c r="G121" t="n">
-        <v>724.5030517578125</v>
+        <v>691.6038208007812</v>
       </c>
       <c r="H121" t="n">
         <v>574.0787976114285</v>
@@ -4305,7 +4305,7 @@
         <v>544.2291194186561</v>
       </c>
       <c r="J121" t="n">
-        <v>579.4617309570312</v>
+        <v>578.2752075195312</v>
       </c>
     </row>
     <row r="122">
@@ -4313,7 +4313,7 @@
         <v>648.0650000000001</v>
       </c>
       <c r="B122" t="n">
-        <v>688.7474365234375</v>
+        <v>689.8055419921875</v>
       </c>
       <c r="C122" t="n">
         <v>679.5013082735761</v>
@@ -4325,10 +4325,10 @@
         <v>640.6887734686733</v>
       </c>
       <c r="F122" t="n">
-        <v>662.3700561523438</v>
+        <v>660.1399536132812</v>
       </c>
       <c r="G122" t="n">
-        <v>684.1193237304688</v>
+        <v>684.815185546875</v>
       </c>
       <c r="H122" t="n">
         <v>665.1589285571429</v>
@@ -4337,7 +4337,7 @@
         <v>616.7612456925369</v>
       </c>
       <c r="J122" t="n">
-        <v>625.3980102539062</v>
+        <v>627.2247314453125</v>
       </c>
     </row>
     <row r="123">
@@ -4345,7 +4345,7 @@
         <v>667.0650000000001</v>
       </c>
       <c r="B123" t="n">
-        <v>696.1204833984375</v>
+        <v>697.241943359375</v>
       </c>
       <c r="C123" t="n">
         <v>687.4007043793565</v>
@@ -4357,10 +4357,10 @@
         <v>644.4807939599481</v>
       </c>
       <c r="F123" t="n">
-        <v>665.80615234375</v>
+        <v>663.1172485351562</v>
       </c>
       <c r="G123" t="n">
-        <v>690.3557739257812</v>
+        <v>692.7693481445312</v>
       </c>
       <c r="H123" t="n">
         <v>680.0520118799998</v>
@@ -4369,7 +4369,7 @@
         <v>660.3544424373293</v>
       </c>
       <c r="J123" t="n">
-        <v>669.0640869140625</v>
+        <v>669.9827270507812</v>
       </c>
     </row>
     <row r="124">
@@ -4377,7 +4377,7 @@
         <v>665.2604167</v>
       </c>
       <c r="B124" t="n">
-        <v>699.5283203125</v>
+        <v>700.6793823242188</v>
       </c>
       <c r="C124" t="n">
         <v>691.0504253649386</v>
@@ -4389,10 +4389,10 @@
         <v>645.3941907720695</v>
       </c>
       <c r="F124" t="n">
-        <v>667.393798828125</v>
+        <v>664.4928588867188</v>
       </c>
       <c r="G124" t="n">
-        <v>693.2371826171875</v>
+        <v>696.4442749023438</v>
       </c>
       <c r="H124" t="n">
         <v>681.1081547571426</v>
@@ -4401,7 +4401,7 @@
         <v>681.889748278818</v>
       </c>
       <c r="J124" t="n">
-        <v>684.6793212890625</v>
+        <v>685.3674926757812</v>
       </c>
     </row>
     <row r="125">
@@ -4409,7 +4409,7 @@
         <v>720.1708333</v>
       </c>
       <c r="B125" t="n">
-        <v>681.4722900390625</v>
+        <v>682.4688110351562</v>
       </c>
       <c r="C125" t="n">
         <v>671.7019045235652</v>
@@ -4421,10 +4421,10 @@
         <v>633.4260155628115</v>
       </c>
       <c r="F125" t="n">
-        <v>658.9774780273438</v>
+        <v>657.2003173828125</v>
       </c>
       <c r="G125" t="n">
-        <v>678.2403564453125</v>
+        <v>676.9619750976562</v>
       </c>
       <c r="H125" t="n">
         <v>661.8066785542856</v>
@@ -4433,7 +4433,7 @@
         <v>676.0332289975989</v>
       </c>
       <c r="J125" t="n">
-        <v>678.1683959960938</v>
+        <v>678.58251953125</v>
       </c>
     </row>
     <row r="126">
@@ -4441,7 +4441,7 @@
         <v>801.2816667</v>
       </c>
       <c r="B126" t="n">
-        <v>840.9076538085938</v>
+        <v>841.8255004882812</v>
       </c>
       <c r="C126" t="n">
         <v>837.3449832806909</v>
@@ -4453,10 +4453,10 @@
         <v>809.2239078506987</v>
       </c>
       <c r="F126" t="n">
-        <v>882.1612548828125</v>
+        <v>880.5689086914062</v>
       </c>
       <c r="G126" t="n">
-        <v>858.6129150390625</v>
+        <v>865.476806640625</v>
       </c>
       <c r="H126" t="n">
         <v>765.8622738028571</v>
@@ -4465,7 +4465,7 @@
         <v>802.661966042533</v>
       </c>
       <c r="J126" t="n">
-        <v>841.9646606445312</v>
+        <v>843.7649536132812</v>
       </c>
     </row>
     <row r="127">
@@ -4473,7 +4473,7 @@
         <v>875.6391667</v>
       </c>
       <c r="B127" t="n">
-        <v>837.5902709960938</v>
+        <v>838.474853515625</v>
       </c>
       <c r="C127" t="n">
         <v>833.8452508287628</v>
@@ -4485,10 +4485,10 @@
         <v>804.3471419903381</v>
       </c>
       <c r="F127" t="n">
-        <v>878.7539672851562</v>
+        <v>877.4170532226562</v>
       </c>
       <c r="G127" t="n">
-        <v>855.4067993164062</v>
+        <v>862.8983154296875</v>
       </c>
       <c r="H127" t="n">
         <v>769.1457619085713</v>
@@ -4497,7 +4497,7 @@
         <v>830.0247513152607</v>
       </c>
       <c r="J127" t="n">
-        <v>826.5073852539062</v>
+        <v>827.5111694335938</v>
       </c>
     </row>
     <row r="128">
@@ -4505,7 +4505,7 @@
         <v>870.6741667</v>
       </c>
       <c r="B128" t="n">
-        <v>845.4105224609375</v>
+        <v>846.3735961914062</v>
       </c>
       <c r="C128" t="n">
         <v>842.094620179736</v>
@@ -4517,10 +4517,10 @@
         <v>813.8384435463255</v>
       </c>
       <c r="F128" t="n">
-        <v>887.424072265625</v>
+        <v>885.7916259765625</v>
       </c>
       <c r="G128" t="n">
-        <v>862.9641723632812</v>
+        <v>868.976318359375</v>
       </c>
       <c r="H128" t="n">
         <v>764.2127381085714</v>
@@ -4529,7 +4529,7 @@
         <v>864.4272198626406</v>
       </c>
       <c r="J128" t="n">
-        <v>875.2625732421875</v>
+        <v>878.1801147460938</v>
       </c>
     </row>
     <row r="129">
@@ -4537,7 +4537,7 @@
         <v>876.3116667</v>
       </c>
       <c r="B129" t="n">
-        <v>861.0556640625</v>
+        <v>862.1798095703125</v>
       </c>
       <c r="C129" t="n">
         <v>858.5933588816824</v>
@@ -4549,10 +4549,10 @@
         <v>827.8752663464282</v>
       </c>
       <c r="F129" t="n">
-        <v>905.7059326171875</v>
+        <v>903.9334106445312</v>
       </c>
       <c r="G129" t="n">
-        <v>878.078857421875</v>
+        <v>881.1319580078125</v>
       </c>
       <c r="H129" t="n">
         <v>771.4536666485715</v>
@@ -4561,7 +4561,7 @@
         <v>871.0845769121526</v>
       </c>
       <c r="J129" t="n">
-        <v>882.944091796875</v>
+        <v>885.7601928710938</v>
       </c>
     </row>
     <row r="130">
@@ -4569,7 +4569,7 @@
         <v>862.6429167</v>
       </c>
       <c r="B130" t="n">
-        <v>864.6593627929688</v>
+        <v>865.8209838867188</v>
       </c>
       <c r="C130" t="n">
         <v>862.3930684009185</v>
@@ -4581,10 +4581,10 @@
         <v>829.4582580992078</v>
       </c>
       <c r="F130" t="n">
-        <v>909.9163818359375</v>
+        <v>908.1115112304688</v>
       </c>
       <c r="G130" t="n">
-        <v>881.1923828125</v>
+        <v>883.931396484375</v>
       </c>
       <c r="H130" t="n">
         <v>767.5565714314287</v>
@@ -4593,7 +4593,7 @@
         <v>871.1800944025749</v>
       </c>
       <c r="J130" t="n">
-        <v>891.9287719726562</v>
+        <v>894.5731201171875</v>
       </c>
     </row>
     <row r="131">
@@ -4601,7 +4601,7 @@
         <v>868.34375</v>
       </c>
       <c r="B131" t="n">
-        <v>871.866455078125</v>
+        <v>873.1045532226562</v>
       </c>
       <c r="C131" t="n">
         <v>869.9924874393907</v>
@@ -4613,10 +4613,10 @@
         <v>828.2552991408896</v>
       </c>
       <c r="F131" t="n">
-        <v>918.5384521484375</v>
+        <v>916.61572265625</v>
       </c>
       <c r="G131" t="n">
-        <v>886.9389038085938</v>
+        <v>889.530029296875</v>
       </c>
       <c r="H131" t="n">
         <v>765.8049047914286</v>
@@ -4625,7 +4625,7 @@
         <v>864.1287069477723</v>
       </c>
       <c r="J131" t="n">
-        <v>884.9959716796875</v>
+        <v>887.2147827148438</v>
       </c>
     </row>
     <row r="132">
@@ -4633,7 +4633,7 @@
         <v>829.2979167</v>
       </c>
       <c r="B132" t="n">
-        <v>875.8966674804688</v>
+        <v>877.1776123046875</v>
       </c>
       <c r="C132" t="n">
         <v>874.2421625595889</v>
@@ -4645,10 +4645,10 @@
         <v>828.4391310057216</v>
       </c>
       <c r="F132" t="n">
-        <v>923.3676147460938</v>
+        <v>921.4435424804688</v>
       </c>
       <c r="G132" t="n">
-        <v>890.1522827148438</v>
+        <v>892.6611938476562</v>
       </c>
       <c r="H132" t="n">
         <v>765.3102381342858</v>
@@ -4657,7 +4657,7 @@
         <v>866.4008812394712</v>
       </c>
       <c r="J132" t="n">
-        <v>892.3861694335938</v>
+        <v>894.6771240234375</v>
       </c>
     </row>
     <row r="133">
@@ -4665,7 +4665,7 @@
         <v>849.6879167</v>
       </c>
       <c r="B133" t="n">
-        <v>875.8018798828125</v>
+        <v>877.0819702148438</v>
       </c>
       <c r="C133" t="n">
         <v>874.1421702038197</v>
@@ -4677,10 +4677,10 @@
         <v>828.4391310057216</v>
       </c>
       <c r="F133" t="n">
-        <v>923.25390625</v>
+        <v>921.3299560546875</v>
       </c>
       <c r="G133" t="n">
-        <v>890.0767822265625</v>
+        <v>892.5875244140625</v>
       </c>
       <c r="H133" t="n">
         <v>765.3102381342858</v>
@@ -4689,7 +4689,7 @@
         <v>848.4234807757841</v>
       </c>
       <c r="J133" t="n">
-        <v>872.0695190429688</v>
+        <v>873.368408203125</v>
       </c>
     </row>
     <row r="134">
@@ -4697,7 +4697,7 @@
         <v>857.2754167000001</v>
       </c>
       <c r="B134" t="n">
-        <v>869.8751831054688</v>
+        <v>871.0919189453125</v>
       </c>
       <c r="C134" t="n">
         <v>867.8926479682339</v>
@@ -4709,10 +4709,10 @@
         <v>827.2538507919486</v>
       </c>
       <c r="F134" t="n">
-        <v>916.1521606445312</v>
+        <v>914.2302856445312</v>
       </c>
       <c r="G134" t="n">
-        <v>885.3509521484375</v>
+        <v>887.9833374023438</v>
       </c>
       <c r="H134" t="n">
         <v>764.32711906</v>
@@ -4721,7 +4721,7 @@
         <v>857.8030401067191</v>
       </c>
       <c r="J134" t="n">
-        <v>880.5001220703125</v>
+        <v>882.3351440429688</v>
       </c>
     </row>
     <row r="135">
@@ -4729,7 +4729,7 @@
         <v>872.4545833</v>
       </c>
       <c r="B135" t="n">
-        <v>865.7500610351562</v>
+        <v>866.9231567382812</v>
       </c>
       <c r="C135" t="n">
         <v>863.5429804922662</v>
@@ -4741,10 +4741,10 @@
         <v>829.4582580992078</v>
       </c>
       <c r="F135" t="n">
-        <v>911.2092895507812</v>
+        <v>909.3759155273438</v>
       </c>
       <c r="G135" t="n">
-        <v>882.061767578125</v>
+        <v>884.778564453125</v>
       </c>
       <c r="H135" t="n">
         <v>766.4073214314285</v>
@@ -4753,7 +4753,7 @@
         <v>860.2673504368669</v>
       </c>
       <c r="J135" t="n">
-        <v>881.1419677734375</v>
+        <v>883.2850952148438</v>
       </c>
     </row>
     <row r="136">
@@ -4761,7 +4761,7 @@
         <v>876.15</v>
       </c>
       <c r="B136" t="n">
-        <v>870.2545166015625</v>
+        <v>871.4752197265625</v>
       </c>
       <c r="C136" t="n">
         <v>868.2926173913113</v>
@@ -4773,10 +4773,10 @@
         <v>828.2552991408896</v>
       </c>
       <c r="F136" t="n">
-        <v>916.606689453125</v>
+        <v>914.6846923828125</v>
       </c>
       <c r="G136" t="n">
-        <v>885.6533203125</v>
+        <v>888.2777709960938</v>
       </c>
       <c r="H136" t="n">
         <v>764.32711906</v>
@@ -4785,7 +4785,7 @@
         <v>870.0459293481158</v>
       </c>
       <c r="J136" t="n">
-        <v>891.8785400390625</v>
+        <v>894.5391235351562</v>
       </c>
     </row>
     <row r="137">
@@ -4793,7 +4793,7 @@
         <v>867.7458333</v>
       </c>
       <c r="B137" t="n">
-        <v>871.96142578125</v>
+        <v>873.2003173828125</v>
       </c>
       <c r="C137" t="n">
         <v>870.0924797951602</v>
@@ -4805,10 +4805,10 @@
         <v>828.2552991408896</v>
       </c>
       <c r="F137" t="n">
-        <v>918.6519775390625</v>
+        <v>916.7293090820312</v>
       </c>
       <c r="G137" t="n">
-        <v>887.0144653320312</v>
+        <v>889.6038818359375</v>
       </c>
       <c r="H137" t="n">
         <v>765.8049047914286</v>
@@ -4817,7 +4817,7 @@
         <v>867.6782782757017</v>
       </c>
       <c r="J137" t="n">
-        <v>896.427734375</v>
+        <v>899.1539916992188</v>
       </c>
     </row>
     <row r="138">
@@ -4825,7 +4825,7 @@
         <v>834.0183333</v>
       </c>
       <c r="B138" t="n">
-        <v>886.3734130859375</v>
+        <v>887.7679443359375</v>
       </c>
       <c r="C138" t="n">
         <v>885.2913178721046</v>
@@ -4837,10 +4837,10 @@
         <v>831.2818565700987</v>
       </c>
       <c r="F138" t="n">
-        <v>935.9236450195312</v>
+        <v>933.9956665039062</v>
       </c>
       <c r="G138" t="n">
-        <v>898.5075073242188</v>
+        <v>900.8018798828125</v>
       </c>
       <c r="H138" t="n">
         <v>769.5737619342858</v>
@@ -4849,7 +4849,7 @@
         <v>869.9598226063266</v>
       </c>
       <c r="J138" t="n">
-        <v>899.5921020507812</v>
+        <v>902.5072631835938</v>
       </c>
     </row>
     <row r="139">
@@ -4857,7 +4857,7 @@
         <v>838.4908333</v>
       </c>
       <c r="B139" t="n">
-        <v>890.41064453125</v>
+        <v>891.8482055664062</v>
       </c>
       <c r="C139" t="n">
         <v>890.3979433346119</v>
@@ -4869,10 +4869,10 @@
         <v>843.4355238572097</v>
       </c>
       <c r="F139" t="n">
-        <v>952.0123291015625</v>
+        <v>950.3880615234375</v>
       </c>
       <c r="G139" t="n">
-        <v>924.3382568359375</v>
+        <v>933.10498046875</v>
       </c>
       <c r="H139" t="n">
         <v>754.5807024</v>
@@ -4881,7 +4881,7 @@
         <v>848.3744939944719</v>
       </c>
       <c r="J139" t="n">
-        <v>889.5702514648438</v>
+        <v>891.0130615234375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>